<commit_message>
chore(admin/attendance): update SF4 blank attendance excel template
</commit_message>
<xml_diff>
--- a/assets/admin/attendance/templates/SF4_Blank.xlsx
+++ b/assets/admin/attendance/templates/SF4_Blank.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\L4T\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\L4T\Documents\Website\ulhs.github.io\assets\admin\attendance\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2E1E8F-AC5D-4F8B-ACEB-698FBC9CD465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F409E2-9757-4606-A183-27CD87CAC7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="month" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="43">
   <si>
     <t>School Form 4 (SF4) Monthly Learner's Movement and Attendance</t>
   </si>
@@ -1270,7 +1270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1594,96 +1594,19 @@
     <xf numFmtId="1" fontId="7" fillId="8" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1696,18 +1619,108 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1966,7 +1979,7 @@
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
-  <dimension ref="A1:AN235"/>
+  <dimension ref="A1:AN236"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="13.54296875" customWidth="1"/>
@@ -1981,134 +1994,134 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A1" s="164" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="112"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="112"/>
-      <c r="L1" s="112"/>
-      <c r="M1" s="112"/>
-      <c r="N1" s="112"/>
-      <c r="O1" s="112"/>
-      <c r="P1" s="112"/>
-      <c r="Q1" s="112"/>
-      <c r="R1" s="112"/>
-      <c r="S1" s="112"/>
-      <c r="T1" s="112"/>
-      <c r="U1" s="112"/>
-      <c r="V1" s="112"/>
-      <c r="W1" s="112"/>
-      <c r="X1" s="112"/>
-      <c r="Y1" s="112"/>
-      <c r="Z1" s="112"/>
-      <c r="AA1" s="112"/>
-      <c r="AB1" s="112"/>
-      <c r="AC1" s="112"/>
-      <c r="AD1" s="112"/>
-      <c r="AE1" s="112"/>
-      <c r="AF1" s="112"/>
-      <c r="AG1" s="112"/>
-      <c r="AH1" s="112"/>
-      <c r="AI1" s="112"/>
-      <c r="AJ1" s="112"/>
-      <c r="AK1" s="112"/>
-      <c r="AL1" s="112"/>
-      <c r="AM1" s="112"/>
-      <c r="AN1" s="112"/>
+      <c r="A1" s="115" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+      <c r="P1" s="116"/>
+      <c r="Q1" s="116"/>
+      <c r="R1" s="116"/>
+      <c r="S1" s="116"/>
+      <c r="T1" s="116"/>
+      <c r="U1" s="116"/>
+      <c r="V1" s="116"/>
+      <c r="W1" s="116"/>
+      <c r="X1" s="116"/>
+      <c r="Y1" s="116"/>
+      <c r="Z1" s="116"/>
+      <c r="AA1" s="116"/>
+      <c r="AB1" s="116"/>
+      <c r="AC1" s="116"/>
+      <c r="AD1" s="116"/>
+      <c r="AE1" s="116"/>
+      <c r="AF1" s="116"/>
+      <c r="AG1" s="116"/>
+      <c r="AH1" s="116"/>
+      <c r="AI1" s="116"/>
+      <c r="AJ1" s="116"/>
+      <c r="AK1" s="116"/>
+      <c r="AL1" s="116"/>
+      <c r="AM1" s="116"/>
+      <c r="AN1" s="116"/>
     </row>
     <row r="2" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A2" s="112"/>
-      <c r="B2" s="112"/>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="112"/>
-      <c r="J2" s="112"/>
-      <c r="K2" s="112"/>
-      <c r="L2" s="112"/>
-      <c r="M2" s="112"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="112"/>
-      <c r="P2" s="112"/>
-      <c r="Q2" s="112"/>
-      <c r="R2" s="112"/>
-      <c r="S2" s="112"/>
-      <c r="T2" s="112"/>
-      <c r="U2" s="112"/>
-      <c r="V2" s="112"/>
-      <c r="W2" s="112"/>
-      <c r="X2" s="112"/>
-      <c r="Y2" s="112"/>
-      <c r="Z2" s="112"/>
-      <c r="AA2" s="112"/>
-      <c r="AB2" s="112"/>
-      <c r="AC2" s="112"/>
-      <c r="AD2" s="112"/>
-      <c r="AE2" s="112"/>
-      <c r="AF2" s="112"/>
-      <c r="AG2" s="112"/>
-      <c r="AH2" s="112"/>
-      <c r="AI2" s="112"/>
-      <c r="AJ2" s="112"/>
-      <c r="AK2" s="112"/>
-      <c r="AL2" s="112"/>
-      <c r="AM2" s="112"/>
-      <c r="AN2" s="112"/>
+      <c r="A2" s="116"/>
+      <c r="B2" s="116"/>
+      <c r="C2" s="116"/>
+      <c r="D2" s="116"/>
+      <c r="E2" s="116"/>
+      <c r="F2" s="116"/>
+      <c r="G2" s="116"/>
+      <c r="H2" s="116"/>
+      <c r="I2" s="116"/>
+      <c r="J2" s="116"/>
+      <c r="K2" s="116"/>
+      <c r="L2" s="116"/>
+      <c r="M2" s="116"/>
+      <c r="N2" s="116"/>
+      <c r="O2" s="116"/>
+      <c r="P2" s="116"/>
+      <c r="Q2" s="116"/>
+      <c r="R2" s="116"/>
+      <c r="S2" s="116"/>
+      <c r="T2" s="116"/>
+      <c r="U2" s="116"/>
+      <c r="V2" s="116"/>
+      <c r="W2" s="116"/>
+      <c r="X2" s="116"/>
+      <c r="Y2" s="116"/>
+      <c r="Z2" s="116"/>
+      <c r="AA2" s="116"/>
+      <c r="AB2" s="116"/>
+      <c r="AC2" s="116"/>
+      <c r="AD2" s="116"/>
+      <c r="AE2" s="116"/>
+      <c r="AF2" s="116"/>
+      <c r="AG2" s="116"/>
+      <c r="AH2" s="116"/>
+      <c r="AI2" s="116"/>
+      <c r="AJ2" s="116"/>
+      <c r="AK2" s="116"/>
+      <c r="AL2" s="116"/>
+      <c r="AM2" s="116"/>
+      <c r="AN2" s="116"/>
     </row>
     <row r="3" spans="1:40" ht="27" customHeight="1">
-      <c r="A3" s="165" t="s">
+      <c r="A3" s="117" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="112"/>
-      <c r="C3" s="112"/>
-      <c r="D3" s="112"/>
-      <c r="E3" s="112"/>
-      <c r="F3" s="112"/>
-      <c r="G3" s="112"/>
-      <c r="H3" s="112"/>
-      <c r="I3" s="112"/>
-      <c r="J3" s="112"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="112"/>
-      <c r="M3" s="112"/>
-      <c r="N3" s="112"/>
-      <c r="O3" s="112"/>
-      <c r="P3" s="112"/>
-      <c r="Q3" s="112"/>
-      <c r="R3" s="112"/>
-      <c r="S3" s="112"/>
-      <c r="T3" s="112"/>
-      <c r="U3" s="112"/>
-      <c r="V3" s="112"/>
-      <c r="W3" s="112"/>
-      <c r="X3" s="112"/>
-      <c r="Y3" s="112"/>
-      <c r="Z3" s="112"/>
-      <c r="AA3" s="112"/>
-      <c r="AB3" s="112"/>
-      <c r="AC3" s="112"/>
-      <c r="AD3" s="112"/>
-      <c r="AE3" s="112"/>
-      <c r="AF3" s="112"/>
-      <c r="AG3" s="112"/>
-      <c r="AH3" s="112"/>
-      <c r="AI3" s="112"/>
-      <c r="AJ3" s="112"/>
-      <c r="AK3" s="112"/>
-      <c r="AL3" s="112"/>
-      <c r="AM3" s="112"/>
-      <c r="AN3" s="112"/>
+      <c r="B3" s="116"/>
+      <c r="C3" s="116"/>
+      <c r="D3" s="116"/>
+      <c r="E3" s="116"/>
+      <c r="F3" s="116"/>
+      <c r="G3" s="116"/>
+      <c r="H3" s="116"/>
+      <c r="I3" s="116"/>
+      <c r="J3" s="116"/>
+      <c r="K3" s="116"/>
+      <c r="L3" s="116"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="116"/>
+      <c r="O3" s="116"/>
+      <c r="P3" s="116"/>
+      <c r="Q3" s="116"/>
+      <c r="R3" s="116"/>
+      <c r="S3" s="116"/>
+      <c r="T3" s="116"/>
+      <c r="U3" s="116"/>
+      <c r="V3" s="116"/>
+      <c r="W3" s="116"/>
+      <c r="X3" s="116"/>
+      <c r="Y3" s="116"/>
+      <c r="Z3" s="116"/>
+      <c r="AA3" s="116"/>
+      <c r="AB3" s="116"/>
+      <c r="AC3" s="116"/>
+      <c r="AD3" s="116"/>
+      <c r="AE3" s="116"/>
+      <c r="AF3" s="116"/>
+      <c r="AG3" s="116"/>
+      <c r="AH3" s="116"/>
+      <c r="AI3" s="116"/>
+      <c r="AJ3" s="116"/>
+      <c r="AK3" s="116"/>
+      <c r="AL3" s="116"/>
+      <c r="AM3" s="116"/>
+      <c r="AN3" s="116"/>
     </row>
     <row r="4" spans="1:40" ht="20.25" customHeight="1">
       <c r="A4" s="1"/>
@@ -2158,41 +2171,41 @@
       <c r="C5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="153"/>
-      <c r="E5" s="133"/>
-      <c r="F5" s="154"/>
-      <c r="G5" s="155" t="s">
+      <c r="D5" s="112"/>
+      <c r="E5" s="113"/>
+      <c r="F5" s="114"/>
+      <c r="G5" s="118" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="156"/>
-      <c r="I5" s="153"/>
-      <c r="J5" s="154"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="112"/>
+      <c r="J5" s="114"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="155" t="s">
+      <c r="L5" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="156"/>
-      <c r="N5" s="153"/>
-      <c r="O5" s="133"/>
-      <c r="P5" s="133"/>
-      <c r="Q5" s="133"/>
-      <c r="R5" s="133"/>
-      <c r="S5" s="133"/>
-      <c r="T5" s="133"/>
-      <c r="U5" s="154"/>
+      <c r="M5" s="119"/>
+      <c r="N5" s="112"/>
+      <c r="O5" s="113"/>
+      <c r="P5" s="113"/>
+      <c r="Q5" s="113"/>
+      <c r="R5" s="113"/>
+      <c r="S5" s="113"/>
+      <c r="T5" s="113"/>
+      <c r="U5" s="114"/>
       <c r="V5" s="2"/>
-      <c r="W5" s="155" t="s">
+      <c r="W5" s="118" t="s">
         <v>5</v>
       </c>
-      <c r="X5" s="156"/>
-      <c r="Y5" s="153"/>
-      <c r="Z5" s="133"/>
-      <c r="AA5" s="133"/>
-      <c r="AB5" s="133"/>
-      <c r="AC5" s="133"/>
-      <c r="AD5" s="133"/>
-      <c r="AE5" s="133"/>
-      <c r="AF5" s="154"/>
+      <c r="X5" s="119"/>
+      <c r="Y5" s="112"/>
+      <c r="Z5" s="113"/>
+      <c r="AA5" s="113"/>
+      <c r="AB5" s="113"/>
+      <c r="AC5" s="113"/>
+      <c r="AD5" s="113"/>
+      <c r="AE5" s="113"/>
+      <c r="AF5" s="114"/>
       <c r="AG5" s="5"/>
       <c r="AH5" s="5"/>
       <c r="AI5" s="5"/>
@@ -2245,52 +2258,52 @@
       <c r="AN6" s="5"/>
     </row>
     <row r="7" spans="1:40" ht="26.25" customHeight="1">
-      <c r="A7" s="155" t="s">
+      <c r="A7" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="156"/>
-      <c r="C7" s="153"/>
-      <c r="D7" s="133"/>
-      <c r="E7" s="133"/>
-      <c r="F7" s="133"/>
-      <c r="G7" s="133"/>
-      <c r="H7" s="133"/>
-      <c r="I7" s="133"/>
-      <c r="J7" s="133"/>
-      <c r="K7" s="133"/>
-      <c r="L7" s="133"/>
-      <c r="M7" s="133"/>
-      <c r="N7" s="133"/>
-      <c r="O7" s="133"/>
-      <c r="P7" s="154"/>
+      <c r="B7" s="119"/>
+      <c r="C7" s="112"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
+      <c r="H7" s="113"/>
+      <c r="I7" s="113"/>
+      <c r="J7" s="113"/>
+      <c r="K7" s="113"/>
+      <c r="L7" s="113"/>
+      <c r="M7" s="113"/>
+      <c r="N7" s="113"/>
+      <c r="O7" s="113"/>
+      <c r="P7" s="114"/>
       <c r="Q7" s="5"/>
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
       <c r="T7" s="5"/>
-      <c r="U7" s="155" t="s">
+      <c r="U7" s="118" t="s">
         <v>7</v>
       </c>
-      <c r="V7" s="112"/>
-      <c r="W7" s="112"/>
-      <c r="X7" s="156"/>
-      <c r="Y7" s="153"/>
-      <c r="Z7" s="133"/>
-      <c r="AA7" s="133"/>
-      <c r="AB7" s="133"/>
-      <c r="AC7" s="154"/>
+      <c r="V7" s="116"/>
+      <c r="W7" s="116"/>
+      <c r="X7" s="119"/>
+      <c r="Y7" s="112"/>
+      <c r="Z7" s="113"/>
+      <c r="AA7" s="113"/>
+      <c r="AB7" s="113"/>
+      <c r="AC7" s="114"/>
       <c r="AD7" s="5"/>
-      <c r="AE7" s="163" t="s">
+      <c r="AE7" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="AF7" s="112"/>
-      <c r="AG7" s="112"/>
-      <c r="AH7" s="112"/>
-      <c r="AI7" s="156"/>
-      <c r="AJ7" s="153"/>
-      <c r="AK7" s="133"/>
-      <c r="AL7" s="133"/>
-      <c r="AM7" s="133"/>
-      <c r="AN7" s="154"/>
+      <c r="AF7" s="116"/>
+      <c r="AG7" s="116"/>
+      <c r="AH7" s="116"/>
+      <c r="AI7" s="119"/>
+      <c r="AJ7" s="112"/>
+      <c r="AK7" s="113"/>
+      <c r="AL7" s="113"/>
+      <c r="AM7" s="113"/>
+      <c r="AN7" s="114"/>
     </row>
     <row r="8" spans="1:40" ht="6.75" customHeight="1">
       <c r="A8" s="1"/>
@@ -2335,132 +2348,132 @@
       <c r="AN8" s="1"/>
     </row>
     <row r="9" spans="1:40" ht="21" customHeight="1">
-      <c r="A9" s="157" t="s">
+      <c r="A9" s="120" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="124" t="s">
+      <c r="B9" s="133" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="124" t="s">
+      <c r="C9" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="125"/>
-      <c r="E9" s="124" t="s">
+      <c r="D9" s="139"/>
+      <c r="E9" s="133" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="125"/>
-      <c r="G9" s="126"/>
-      <c r="H9" s="137" t="s">
+      <c r="F9" s="139"/>
+      <c r="G9" s="157"/>
+      <c r="H9" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="138"/>
-      <c r="J9" s="138"/>
-      <c r="K9" s="138"/>
-      <c r="L9" s="138"/>
-      <c r="M9" s="138"/>
-      <c r="N9" s="139" t="s">
+      <c r="I9" s="127"/>
+      <c r="J9" s="127"/>
+      <c r="K9" s="127"/>
+      <c r="L9" s="127"/>
+      <c r="M9" s="127"/>
+      <c r="N9" s="130" t="s">
         <v>14</v>
       </c>
-      <c r="O9" s="138"/>
-      <c r="P9" s="138"/>
-      <c r="Q9" s="138"/>
-      <c r="R9" s="138"/>
-      <c r="S9" s="138"/>
-      <c r="T9" s="138"/>
-      <c r="U9" s="138"/>
-      <c r="V9" s="140"/>
-      <c r="W9" s="137" t="s">
+      <c r="O9" s="127"/>
+      <c r="P9" s="127"/>
+      <c r="Q9" s="127"/>
+      <c r="R9" s="127"/>
+      <c r="S9" s="127"/>
+      <c r="T9" s="127"/>
+      <c r="U9" s="127"/>
+      <c r="V9" s="128"/>
+      <c r="W9" s="145" t="s">
         <v>15</v>
       </c>
-      <c r="X9" s="138"/>
-      <c r="Y9" s="138"/>
-      <c r="Z9" s="138"/>
-      <c r="AA9" s="138"/>
-      <c r="AB9" s="138"/>
-      <c r="AC9" s="138"/>
-      <c r="AD9" s="138"/>
-      <c r="AE9" s="138"/>
-      <c r="AF9" s="139" t="s">
+      <c r="X9" s="127"/>
+      <c r="Y9" s="127"/>
+      <c r="Z9" s="127"/>
+      <c r="AA9" s="127"/>
+      <c r="AB9" s="127"/>
+      <c r="AC9" s="127"/>
+      <c r="AD9" s="127"/>
+      <c r="AE9" s="127"/>
+      <c r="AF9" s="130" t="s">
         <v>16</v>
       </c>
-      <c r="AG9" s="138"/>
-      <c r="AH9" s="138"/>
-      <c r="AI9" s="138"/>
-      <c r="AJ9" s="138"/>
-      <c r="AK9" s="138"/>
-      <c r="AL9" s="138"/>
-      <c r="AM9" s="138"/>
-      <c r="AN9" s="140"/>
+      <c r="AG9" s="127"/>
+      <c r="AH9" s="127"/>
+      <c r="AI9" s="127"/>
+      <c r="AJ9" s="127"/>
+      <c r="AK9" s="127"/>
+      <c r="AL9" s="127"/>
+      <c r="AM9" s="127"/>
+      <c r="AN9" s="128"/>
     </row>
     <row r="10" spans="1:40" ht="60.75" customHeight="1">
-      <c r="A10" s="158"/>
-      <c r="B10" s="127"/>
-      <c r="C10" s="127"/>
-      <c r="D10" s="112"/>
-      <c r="E10" s="127"/>
-      <c r="F10" s="112"/>
-      <c r="G10" s="128"/>
-      <c r="H10" s="129" t="s">
+      <c r="A10" s="121"/>
+      <c r="B10" s="134"/>
+      <c r="C10" s="134"/>
+      <c r="D10" s="116"/>
+      <c r="E10" s="134"/>
+      <c r="F10" s="116"/>
+      <c r="G10" s="158"/>
+      <c r="H10" s="159" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="118"/>
-      <c r="J10" s="121"/>
-      <c r="K10" s="114" t="s">
+      <c r="I10" s="147"/>
+      <c r="J10" s="149"/>
+      <c r="K10" s="154" t="s">
         <v>18</v>
       </c>
-      <c r="L10" s="115"/>
-      <c r="M10" s="116"/>
-      <c r="N10" s="120" t="s">
+      <c r="L10" s="144"/>
+      <c r="M10" s="151"/>
+      <c r="N10" s="150" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="115"/>
-      <c r="P10" s="116"/>
-      <c r="Q10" s="117" t="s">
+      <c r="O10" s="144"/>
+      <c r="P10" s="151"/>
+      <c r="Q10" s="146" t="s">
         <v>20</v>
       </c>
-      <c r="R10" s="118"/>
-      <c r="S10" s="121"/>
-      <c r="T10" s="117" t="s">
+      <c r="R10" s="147"/>
+      <c r="S10" s="149"/>
+      <c r="T10" s="146" t="s">
         <v>21</v>
       </c>
-      <c r="U10" s="118"/>
-      <c r="V10" s="119"/>
-      <c r="W10" s="120" t="s">
+      <c r="U10" s="147"/>
+      <c r="V10" s="148"/>
+      <c r="W10" s="150" t="s">
         <v>19</v>
       </c>
-      <c r="X10" s="115"/>
-      <c r="Y10" s="116"/>
-      <c r="Z10" s="117" t="s">
+      <c r="X10" s="144"/>
+      <c r="Y10" s="151"/>
+      <c r="Z10" s="146" t="s">
         <v>20</v>
       </c>
-      <c r="AA10" s="118"/>
-      <c r="AB10" s="121"/>
-      <c r="AC10" s="117" t="s">
+      <c r="AA10" s="147"/>
+      <c r="AB10" s="149"/>
+      <c r="AC10" s="146" t="s">
         <v>21</v>
       </c>
-      <c r="AD10" s="118"/>
-      <c r="AE10" s="119"/>
-      <c r="AF10" s="120" t="s">
+      <c r="AD10" s="147"/>
+      <c r="AE10" s="148"/>
+      <c r="AF10" s="150" t="s">
         <v>19</v>
       </c>
-      <c r="AG10" s="115"/>
-      <c r="AH10" s="116"/>
-      <c r="AI10" s="117" t="s">
+      <c r="AG10" s="144"/>
+      <c r="AH10" s="151"/>
+      <c r="AI10" s="146" t="s">
         <v>20</v>
       </c>
-      <c r="AJ10" s="118"/>
-      <c r="AK10" s="121"/>
-      <c r="AL10" s="117" t="s">
+      <c r="AJ10" s="147"/>
+      <c r="AK10" s="149"/>
+      <c r="AL10" s="146" t="s">
         <v>21</v>
       </c>
-      <c r="AM10" s="118"/>
-      <c r="AN10" s="119"/>
+      <c r="AM10" s="147"/>
+      <c r="AN10" s="148"/>
     </row>
     <row r="11" spans="1:40" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A11" s="159"/>
-      <c r="B11" s="143"/>
-      <c r="C11" s="143"/>
-      <c r="D11" s="148"/>
+      <c r="A11" s="122"/>
+      <c r="B11" s="135"/>
+      <c r="C11" s="135"/>
+      <c r="D11" s="124"/>
       <c r="E11" s="7" t="s">
         <v>22</v>
       </c>
@@ -2575,24 +2588,24 @@
         <v>25</v>
       </c>
       <c r="B12" s="12"/>
-      <c r="C12" s="149"/>
-      <c r="D12" s="150"/>
+      <c r="C12" s="140"/>
+      <c r="D12" s="141"/>
       <c r="E12" s="13"/>
       <c r="F12" s="14"/>
       <c r="G12" s="15">
-        <f t="shared" ref="G12:G17" si="0">SUM(E12:F12)</f>
+        <f t="shared" ref="G12:G18" si="0">SUM(E12:F12)</f>
         <v>0</v>
       </c>
       <c r="H12" s="16"/>
       <c r="I12" s="17"/>
       <c r="J12" s="17">
-        <f t="shared" ref="J12:J17" si="1">SUM(H12:I12)</f>
+        <f t="shared" ref="J12:J18" si="1">SUM(H12:I12)</f>
         <v>0</v>
       </c>
       <c r="K12" s="17"/>
       <c r="L12" s="17"/>
       <c r="M12" s="86" t="e">
-        <f t="shared" ref="M12:M17" si="2">AVERAGE(K12:L12)</f>
+        <f t="shared" ref="M12:M18" si="2">AVERAGE(K12:L12)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="N12" s="94">
@@ -2682,8 +2695,8 @@
         <v>25</v>
       </c>
       <c r="B13" s="82"/>
-      <c r="C13" s="134"/>
-      <c r="D13" s="135"/>
+      <c r="C13" s="163"/>
+      <c r="D13" s="164"/>
       <c r="E13" s="83"/>
       <c r="F13" s="84"/>
       <c r="G13" s="85">
@@ -2789,8 +2802,8 @@
         <v>26</v>
       </c>
       <c r="B14" s="23"/>
-      <c r="C14" s="151"/>
-      <c r="D14" s="145"/>
+      <c r="C14" s="131"/>
+      <c r="D14" s="132"/>
       <c r="E14" s="24"/>
       <c r="F14" s="25"/>
       <c r="G14" s="26">
@@ -2896,8 +2909,8 @@
         <v>26</v>
       </c>
       <c r="B15" s="23"/>
-      <c r="C15" s="151"/>
-      <c r="D15" s="145"/>
+      <c r="C15" s="131"/>
+      <c r="D15" s="132"/>
       <c r="E15" s="24"/>
       <c r="F15" s="25"/>
       <c r="G15" s="26">
@@ -3003,8 +3016,8 @@
         <v>27</v>
       </c>
       <c r="B16" s="34"/>
-      <c r="C16" s="152"/>
-      <c r="D16" s="145"/>
+      <c r="C16" s="142"/>
+      <c r="D16" s="132"/>
       <c r="E16" s="35"/>
       <c r="F16" s="36"/>
       <c r="G16" s="37">
@@ -3105,884 +3118,947 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:40" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A17" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="39"/>
-      <c r="C17" s="144"/>
-      <c r="D17" s="145"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="42">
+    <row r="17" spans="1:40" s="111" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A17" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="34"/>
+      <c r="C17" s="142"/>
+      <c r="D17" s="132"/>
+      <c r="E17" s="167"/>
+      <c r="F17" s="168"/>
+      <c r="G17" s="37">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H17" s="43"/>
-      <c r="I17" s="44"/>
-      <c r="J17" s="44">
+      <c r="H17" s="169"/>
+      <c r="I17" s="170"/>
+      <c r="J17" s="28">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K17" s="44"/>
-      <c r="L17" s="44"/>
-      <c r="M17" s="89" t="e">
+      <c r="K17" s="170"/>
+      <c r="L17" s="170"/>
+      <c r="M17" s="88" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N17" s="102">
-        <v>0</v>
-      </c>
-      <c r="O17" s="103">
-        <v>0</v>
-      </c>
-      <c r="P17" s="103">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="103">
-        <v>0</v>
-      </c>
-      <c r="R17" s="103">
-        <v>0</v>
-      </c>
-      <c r="S17" s="103">
-        <v>0</v>
-      </c>
-      <c r="T17" s="103">
-        <v>0</v>
-      </c>
-      <c r="U17" s="103">
-        <v>0</v>
-      </c>
-      <c r="V17" s="104">
-        <v>0</v>
-      </c>
-      <c r="W17" s="105">
-        <v>0</v>
-      </c>
-      <c r="X17" s="103">
-        <v>0</v>
-      </c>
-      <c r="Y17" s="103">
-        <v>0</v>
-      </c>
-      <c r="Z17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AC17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AD17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AE17" s="104">
-        <v>0</v>
-      </c>
-      <c r="AF17" s="106">
-        <v>0</v>
-      </c>
-      <c r="AG17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AH17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AI17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AJ17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AK17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AL17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AM17" s="103">
-        <v>0</v>
-      </c>
-      <c r="AN17" s="107">
+      <c r="N17" s="100">
+        <v>0</v>
+      </c>
+      <c r="O17" s="30">
+        <v>0</v>
+      </c>
+      <c r="P17" s="30">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="30">
+        <v>0</v>
+      </c>
+      <c r="R17" s="30">
+        <v>0</v>
+      </c>
+      <c r="S17" s="30">
+        <v>0</v>
+      </c>
+      <c r="T17" s="30">
+        <v>0</v>
+      </c>
+      <c r="U17" s="30">
+        <v>0</v>
+      </c>
+      <c r="V17" s="31">
+        <v>0</v>
+      </c>
+      <c r="W17" s="32">
+        <v>0</v>
+      </c>
+      <c r="X17" s="30">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="30">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AD17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="31">
+        <v>0</v>
+      </c>
+      <c r="AF17" s="93">
+        <v>0</v>
+      </c>
+      <c r="AG17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AH17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AI17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AJ17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AK17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AL17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AM17" s="30">
+        <v>0</v>
+      </c>
+      <c r="AN17" s="101">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:40" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A18" s="162" t="s">
+      <c r="A18" s="38" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="39"/>
+      <c r="C18" s="136"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="42">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H18" s="43"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="44">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K18" s="44"/>
+      <c r="L18" s="44"/>
+      <c r="M18" s="89" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="N18" s="102">
+        <v>0</v>
+      </c>
+      <c r="O18" s="103">
+        <v>0</v>
+      </c>
+      <c r="P18" s="103">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="103">
+        <v>0</v>
+      </c>
+      <c r="R18" s="103">
+        <v>0</v>
+      </c>
+      <c r="S18" s="103">
+        <v>0</v>
+      </c>
+      <c r="T18" s="103">
+        <v>0</v>
+      </c>
+      <c r="U18" s="103">
+        <v>0</v>
+      </c>
+      <c r="V18" s="104">
+        <v>0</v>
+      </c>
+      <c r="W18" s="105">
+        <v>0</v>
+      </c>
+      <c r="X18" s="103">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="103">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="104">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="106">
+        <v>0</v>
+      </c>
+      <c r="AG18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AI18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AK18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AL18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AM18" s="103">
+        <v>0</v>
+      </c>
+      <c r="AN18" s="107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:40" ht="19.5" customHeight="1" thickBot="1">
+      <c r="A19" s="126" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="138"/>
-      <c r="C18" s="138"/>
-      <c r="D18" s="140"/>
-      <c r="E18" s="160"/>
-      <c r="F18" s="148"/>
-      <c r="G18" s="148"/>
-      <c r="H18" s="148"/>
-      <c r="I18" s="148"/>
-      <c r="J18" s="148"/>
-      <c r="K18" s="148"/>
-      <c r="L18" s="148"/>
-      <c r="M18" s="148"/>
-      <c r="N18" s="148"/>
-      <c r="O18" s="148"/>
-      <c r="P18" s="148"/>
-      <c r="Q18" s="148"/>
-      <c r="R18" s="148"/>
-      <c r="S18" s="148"/>
-      <c r="T18" s="148"/>
-      <c r="U18" s="148"/>
-      <c r="V18" s="148"/>
-      <c r="W18" s="148"/>
-      <c r="X18" s="148"/>
-      <c r="Y18" s="148"/>
-      <c r="Z18" s="148"/>
-      <c r="AA18" s="148"/>
-      <c r="AB18" s="148"/>
-      <c r="AC18" s="148"/>
-      <c r="AD18" s="148"/>
-      <c r="AE18" s="148"/>
-      <c r="AF18" s="148"/>
-      <c r="AG18" s="148"/>
-      <c r="AH18" s="148"/>
-      <c r="AI18" s="148"/>
-      <c r="AJ18" s="148"/>
-      <c r="AK18" s="148"/>
-      <c r="AL18" s="148"/>
-      <c r="AM18" s="148"/>
-      <c r="AN18" s="161"/>
-    </row>
-    <row r="19" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A19" s="130" t="str">
+      <c r="B19" s="127"/>
+      <c r="C19" s="127"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="123"/>
+      <c r="F19" s="124"/>
+      <c r="G19" s="124"/>
+      <c r="H19" s="124"/>
+      <c r="I19" s="124"/>
+      <c r="J19" s="124"/>
+      <c r="K19" s="124"/>
+      <c r="L19" s="124"/>
+      <c r="M19" s="124"/>
+      <c r="N19" s="124"/>
+      <c r="O19" s="124"/>
+      <c r="P19" s="124"/>
+      <c r="Q19" s="124"/>
+      <c r="R19" s="124"/>
+      <c r="S19" s="124"/>
+      <c r="T19" s="124"/>
+      <c r="U19" s="124"/>
+      <c r="V19" s="124"/>
+      <c r="W19" s="124"/>
+      <c r="X19" s="124"/>
+      <c r="Y19" s="124"/>
+      <c r="Z19" s="124"/>
+      <c r="AA19" s="124"/>
+      <c r="AB19" s="124"/>
+      <c r="AC19" s="124"/>
+      <c r="AD19" s="124"/>
+      <c r="AE19" s="124"/>
+      <c r="AF19" s="124"/>
+      <c r="AG19" s="124"/>
+      <c r="AH19" s="124"/>
+      <c r="AI19" s="124"/>
+      <c r="AJ19" s="124"/>
+      <c r="AK19" s="124"/>
+      <c r="AL19" s="124"/>
+      <c r="AM19" s="124"/>
+      <c r="AN19" s="125"/>
+    </row>
+    <row r="20" spans="1:40" ht="19.5" customHeight="1">
+      <c r="A20" s="160" t="str">
         <f>A12</f>
         <v>Grade 7 (I)</v>
       </c>
-      <c r="B19" s="131"/>
-      <c r="C19" s="131"/>
-      <c r="D19" s="131"/>
-      <c r="E19" s="45">
+      <c r="B20" s="161"/>
+      <c r="C20" s="161"/>
+      <c r="D20" s="161"/>
+      <c r="E20" s="45">
         <f>SUM(E12:E13)</f>
         <v>0</v>
       </c>
-      <c r="F19" s="46">
+      <c r="F20" s="46">
         <f>SUM(F12:F13)</f>
         <v>0</v>
       </c>
-      <c r="G19" s="47">
-        <f>SUM(E19:F19)</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="48">
-        <f t="shared" ref="H19:I19" si="6">SUM(H12:H13)</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="49">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J19" s="49">
-        <f>SUM(H19:I19)</f>
-        <v>0</v>
-      </c>
-      <c r="K19" s="49" t="e">
+      <c r="G20" s="47">
+        <f>SUM(E20:F20)</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="48">
+        <f>SUM(H12:H13)</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="49">
+        <f>SUM(I12:I13)</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="49">
+        <f>SUM(H20:I20)</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="49" t="e">
         <f>AVERAGE(K12:K13)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L19" s="49" t="e">
+      <c r="L20" s="49" t="e">
         <f>AVERAGE(L12:L13)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M19" s="50" t="e">
-        <f t="shared" ref="M19:M23" si="7">AVERAGE(K19:L19)</f>
+      <c r="M20" s="50" t="e">
+        <f t="shared" ref="M20:M24" si="6">AVERAGE(K20:L20)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="N19" s="18">
-        <v>0</v>
-      </c>
-      <c r="O19" s="19">
-        <v>0</v>
-      </c>
-      <c r="P19" s="19">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="19">
-        <v>0</v>
-      </c>
-      <c r="R19" s="19">
-        <v>0</v>
-      </c>
-      <c r="S19" s="19">
-        <v>0</v>
-      </c>
-      <c r="T19" s="19">
-        <v>0</v>
-      </c>
-      <c r="U19" s="19">
-        <v>0</v>
-      </c>
-      <c r="V19" s="20">
-        <v>0</v>
-      </c>
-      <c r="W19" s="21">
-        <v>0</v>
-      </c>
-      <c r="X19" s="19">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="19">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AC19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AD19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AE19" s="20">
-        <v>0</v>
-      </c>
-      <c r="AF19" s="18">
-        <v>0</v>
-      </c>
-      <c r="AG19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AH19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AI19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AJ19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AK19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AL19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AM19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AN19" s="20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A20" s="132" t="s">
+      <c r="N20" s="18">
+        <v>0</v>
+      </c>
+      <c r="O20" s="19">
+        <v>0</v>
+      </c>
+      <c r="P20" s="19">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="19">
+        <v>0</v>
+      </c>
+      <c r="R20" s="19">
+        <v>0</v>
+      </c>
+      <c r="S20" s="19">
+        <v>0</v>
+      </c>
+      <c r="T20" s="19">
+        <v>0</v>
+      </c>
+      <c r="U20" s="19">
+        <v>0</v>
+      </c>
+      <c r="V20" s="20">
+        <v>0</v>
+      </c>
+      <c r="W20" s="21">
+        <v>0</v>
+      </c>
+      <c r="X20" s="19">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="19">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="20">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="18">
+        <v>0</v>
+      </c>
+      <c r="AG20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AH20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AI20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AJ20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AK20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AL20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AM20" s="19">
+        <v>0</v>
+      </c>
+      <c r="AN20" s="20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:40" ht="19.5" customHeight="1">
+      <c r="A21" s="162" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="133"/>
-      <c r="C20" s="133"/>
-      <c r="D20" s="133"/>
-      <c r="E20" s="51">
+      <c r="B21" s="113"/>
+      <c r="C21" s="113"/>
+      <c r="D21" s="113"/>
+      <c r="E21" s="51">
         <f>E14+E15</f>
         <v>0</v>
       </c>
-      <c r="F20" s="52">
+      <c r="F21" s="52">
         <f>F14+F15</f>
         <v>0</v>
       </c>
-      <c r="G20" s="53">
-        <f t="shared" ref="G20" si="8">SUM(E20:F20)</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="54">
-        <f t="shared" ref="E20:L20" si="9">H15</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="55">
+      <c r="G21" s="53">
+        <f t="shared" ref="G21" si="7">SUM(E21:F21)</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="54">
+        <f>H15</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="55">
+        <f>I15</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="55">
+        <f>J15</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="55">
+        <f>K15</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="55">
+        <f>L15</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="56">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N21" s="29">
+        <v>0</v>
+      </c>
+      <c r="O21" s="30">
+        <v>0</v>
+      </c>
+      <c r="P21" s="30">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="30">
+        <v>0</v>
+      </c>
+      <c r="R21" s="30">
+        <v>0</v>
+      </c>
+      <c r="S21" s="30">
+        <v>0</v>
+      </c>
+      <c r="T21" s="30">
+        <v>0</v>
+      </c>
+      <c r="U21" s="30">
+        <v>0</v>
+      </c>
+      <c r="V21" s="31">
+        <v>0</v>
+      </c>
+      <c r="W21" s="32">
+        <v>0</v>
+      </c>
+      <c r="X21" s="30">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="30">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="31">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="29">
+        <v>0</v>
+      </c>
+      <c r="AG21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AH21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AI21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AK21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AL21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AM21" s="30">
+        <v>0</v>
+      </c>
+      <c r="AN21" s="31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:40" ht="19.5" customHeight="1">
+      <c r="A22" s="165" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="113"/>
+      <c r="C22" s="113"/>
+      <c r="D22" s="113"/>
+      <c r="E22" s="57">
+        <f t="shared" ref="E22:L22" si="8">E16</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="58">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G22" s="59">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="H22" s="54">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I22" s="55">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J22" s="55">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="K22" s="55">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="L22" s="55">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="M22" s="56">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N22" s="29">
+        <v>0</v>
+      </c>
+      <c r="O22" s="30">
+        <v>0</v>
+      </c>
+      <c r="P22" s="30">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="30">
+        <v>0</v>
+      </c>
+      <c r="R22" s="30">
+        <v>0</v>
+      </c>
+      <c r="S22" s="30">
+        <v>0</v>
+      </c>
+      <c r="T22" s="30">
+        <v>0</v>
+      </c>
+      <c r="U22" s="30">
+        <v>0</v>
+      </c>
+      <c r="V22" s="31">
+        <v>0</v>
+      </c>
+      <c r="W22" s="32">
+        <v>0</v>
+      </c>
+      <c r="X22" s="30">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="30">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="31">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="29">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AI22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AJ22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AK22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AL22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AM22" s="30">
+        <v>0</v>
+      </c>
+      <c r="AN22" s="31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:40" ht="19.5" customHeight="1">
+      <c r="A23" s="166" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="113"/>
+      <c r="C23" s="113"/>
+      <c r="D23" s="113"/>
+      <c r="E23" s="60">
+        <f t="shared" ref="E23:L23" si="9">E18</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="61">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J20" s="55">
+      <c r="G23" s="62">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="K20" s="55">
+      <c r="H23" s="54">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="L20" s="55">
+      <c r="I23" s="55">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="M20" s="56">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="N20" s="29">
-        <v>0</v>
-      </c>
-      <c r="O20" s="30">
-        <v>0</v>
-      </c>
-      <c r="P20" s="30">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="30">
-        <v>0</v>
-      </c>
-      <c r="R20" s="30">
-        <v>0</v>
-      </c>
-      <c r="S20" s="30">
-        <v>0</v>
-      </c>
-      <c r="T20" s="30">
-        <v>0</v>
-      </c>
-      <c r="U20" s="30">
-        <v>0</v>
-      </c>
-      <c r="V20" s="31">
-        <v>0</v>
-      </c>
-      <c r="W20" s="32">
-        <v>0</v>
-      </c>
-      <c r="X20" s="30">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="30">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AC20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AD20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AE20" s="31">
-        <v>0</v>
-      </c>
-      <c r="AF20" s="29">
-        <v>0</v>
-      </c>
-      <c r="AG20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AH20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AI20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AJ20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AK20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AL20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AM20" s="30">
-        <v>0</v>
-      </c>
-      <c r="AN20" s="31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A21" s="141" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="133"/>
-      <c r="C21" s="133"/>
-      <c r="D21" s="133"/>
-      <c r="E21" s="57">
-        <f t="shared" ref="E21:L21" si="10">E16</f>
-        <v>0</v>
-      </c>
-      <c r="F21" s="58">
+      <c r="J23" s="55">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="K23" s="55">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="L23" s="55">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="M23" s="56">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N23" s="29">
+        <v>0</v>
+      </c>
+      <c r="O23" s="30">
+        <v>0</v>
+      </c>
+      <c r="P23" s="30">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="30">
+        <v>0</v>
+      </c>
+      <c r="R23" s="30">
+        <v>0</v>
+      </c>
+      <c r="S23" s="30">
+        <v>0</v>
+      </c>
+      <c r="T23" s="30">
+        <v>0</v>
+      </c>
+      <c r="U23" s="30">
+        <v>0</v>
+      </c>
+      <c r="V23" s="31">
+        <v>0</v>
+      </c>
+      <c r="W23" s="32">
+        <v>0</v>
+      </c>
+      <c r="X23" s="30">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="30">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="31">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="29">
+        <v>0</v>
+      </c>
+      <c r="AG23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AI23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AJ23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AK23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AL23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AM23" s="30">
+        <v>0</v>
+      </c>
+      <c r="AN23" s="31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:40" ht="19.5" customHeight="1">
+      <c r="A24" s="137" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="138"/>
+      <c r="C24" s="138"/>
+      <c r="D24" s="138"/>
+      <c r="E24" s="108">
+        <f t="shared" ref="E24:J24" si="10">SUM(E20:E23)</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="109">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="G21" s="59">
+      <c r="G24" s="110">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="H21" s="54">
+      <c r="H24" s="63">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="I21" s="55">
+      <c r="I24" s="64">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J21" s="55">
+      <c r="J24" s="64">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="K21" s="55">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="L21" s="55">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="M21" s="56">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="N21" s="29">
-        <v>0</v>
-      </c>
-      <c r="O21" s="30">
-        <v>0</v>
-      </c>
-      <c r="P21" s="30">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="30">
-        <v>0</v>
-      </c>
-      <c r="R21" s="30">
-        <v>0</v>
-      </c>
-      <c r="S21" s="30">
-        <v>0</v>
-      </c>
-      <c r="T21" s="30">
-        <v>0</v>
-      </c>
-      <c r="U21" s="30">
-        <v>0</v>
-      </c>
-      <c r="V21" s="31">
-        <v>0</v>
-      </c>
-      <c r="W21" s="32">
-        <v>0</v>
-      </c>
-      <c r="X21" s="30">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="30">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AC21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AD21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AE21" s="31">
-        <v>0</v>
-      </c>
-      <c r="AF21" s="29">
-        <v>0</v>
-      </c>
-      <c r="AG21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AH21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AI21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AJ21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AK21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AL21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AM21" s="30">
-        <v>0</v>
-      </c>
-      <c r="AN21" s="31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A22" s="142" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="133"/>
-      <c r="C22" s="133"/>
-      <c r="D22" s="133"/>
-      <c r="E22" s="60">
-        <f t="shared" ref="E22:L22" si="11">E17</f>
-        <v>0</v>
-      </c>
-      <c r="F22" s="61">
+      <c r="K24" s="64" t="e">
+        <f t="shared" ref="K24:L24" si="11">AVERAGE(K20:K23)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L24" s="64" t="e">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="G22" s="62">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="H22" s="54">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I22" s="55">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J22" s="55">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="K22" s="55">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="L22" s="55">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="M22" s="56">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="N22" s="29">
-        <v>0</v>
-      </c>
-      <c r="O22" s="30">
-        <v>0</v>
-      </c>
-      <c r="P22" s="30">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="30">
-        <v>0</v>
-      </c>
-      <c r="R22" s="30">
-        <v>0</v>
-      </c>
-      <c r="S22" s="30">
-        <v>0</v>
-      </c>
-      <c r="T22" s="30">
-        <v>0</v>
-      </c>
-      <c r="U22" s="30">
-        <v>0</v>
-      </c>
-      <c r="V22" s="31">
-        <v>0</v>
-      </c>
-      <c r="W22" s="32">
-        <v>0</v>
-      </c>
-      <c r="X22" s="30">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="30">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AE22" s="31">
-        <v>0</v>
-      </c>
-      <c r="AF22" s="29">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AH22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AI22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AJ22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AK22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AL22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AM22" s="30">
-        <v>0</v>
-      </c>
-      <c r="AN22" s="31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A23" s="146" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="147"/>
-      <c r="C23" s="147"/>
-      <c r="D23" s="147"/>
-      <c r="E23" s="108">
-        <f t="shared" ref="E23:J23" si="12">SUM(E19:E22)</f>
-        <v>0</v>
-      </c>
-      <c r="F23" s="109">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M24" s="65" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="N24" s="66">
+        <f t="shared" ref="N24:AN24" si="12">SUM(N20:N23)</f>
+        <v>0</v>
+      </c>
+      <c r="O24" s="67">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="G23" s="110">
+      <c r="P24" s="67">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="H23" s="63">
+      <c r="Q24" s="67">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="I23" s="64">
+      <c r="R24" s="67">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J23" s="64">
+      <c r="S24" s="67">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="K23" s="64" t="e">
-        <f t="shared" ref="K23:L23" si="13">AVERAGE(K19:K22)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L23" s="64" t="e">
-        <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M23" s="65" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N23" s="66">
-        <f t="shared" ref="N23:AN23" si="14">SUM(N19:N22)</f>
-        <v>0</v>
-      </c>
-      <c r="O23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="P23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="Q23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="R23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="S23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="T23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="U23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="V23" s="68">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="W23" s="69">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="X23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="Y23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="Z23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AA23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AB23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AC23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AD23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AE23" s="68">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AF23" s="66">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AG23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AH23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AI23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AJ23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AK23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AL23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AM23" s="67">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AN23" s="68">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A24" s="70" t="s">
+      <c r="T24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="V24" s="68">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="W24" s="69">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="X24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="Y24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="Z24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AA24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AB24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AC24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AD24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AE24" s="68">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AF24" s="66">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AG24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AH24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AI24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AJ24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AK24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AL24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AM24" s="67">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AN24" s="68">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:40" ht="16.5" customHeight="1">
+      <c r="A25" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="71"/>
-      <c r="C24" s="71"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
-      <c r="R24" s="1"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="1"/>
-      <c r="U24" s="1"/>
-      <c r="V24" s="1"/>
-      <c r="W24" s="1"/>
-      <c r="X24" s="1"/>
-      <c r="Y24" s="72" t="s">
-        <v>32</v>
-      </c>
-      <c r="Z24" s="1"/>
-      <c r="AA24" s="1"/>
-      <c r="AB24" s="1"/>
-      <c r="AC24" s="1"/>
-      <c r="AD24" s="1"/>
-      <c r="AE24" s="1"/>
-      <c r="AF24" s="1"/>
-      <c r="AG24" s="1"/>
-      <c r="AH24" s="1"/>
-      <c r="AI24" s="1"/>
-      <c r="AJ24" s="1"/>
-      <c r="AK24" s="1"/>
-      <c r="AL24" s="1"/>
-      <c r="AM24" s="1"/>
-      <c r="AN24" s="1"/>
-    </row>
-    <row r="25" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A25" s="113" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" s="112"/>
-      <c r="C25" s="112"/>
-      <c r="D25" s="112"/>
-      <c r="E25" s="112"/>
-      <c r="F25" s="112"/>
-      <c r="G25" s="112"/>
-      <c r="H25" s="112"/>
-      <c r="I25" s="112"/>
-      <c r="J25" s="112"/>
-      <c r="K25" s="112"/>
-      <c r="L25" s="112"/>
-      <c r="M25" s="112"/>
-      <c r="N25" s="112"/>
-      <c r="O25" s="112"/>
-      <c r="P25" s="112"/>
-      <c r="Q25" s="112"/>
-      <c r="R25" s="112"/>
-      <c r="S25" s="112"/>
-      <c r="T25" s="112"/>
-      <c r="U25" s="112"/>
-      <c r="V25" s="112"/>
+      <c r="B25" s="71"/>
+      <c r="C25" s="71"/>
+      <c r="D25" s="71"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
+      <c r="T25" s="1"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="1"/>
       <c r="W25" s="1"/>
       <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
+      <c r="Y25" s="72" t="s">
+        <v>32</v>
+      </c>
       <c r="Z25" s="1"/>
       <c r="AA25" s="1"/>
       <c r="AB25" s="1"/>
@@ -4000,51 +4076,53 @@
       <c r="AN25" s="1"/>
     </row>
     <row r="26" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="153" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="116"/>
+      <c r="C26" s="116"/>
+      <c r="D26" s="116"/>
+      <c r="E26" s="116"/>
+      <c r="F26" s="116"/>
+      <c r="G26" s="116"/>
+      <c r="H26" s="116"/>
+      <c r="I26" s="116"/>
+      <c r="J26" s="116"/>
+      <c r="K26" s="116"/>
+      <c r="L26" s="116"/>
+      <c r="M26" s="116"/>
+      <c r="N26" s="116"/>
+      <c r="O26" s="116"/>
+      <c r="P26" s="116"/>
+      <c r="Q26" s="116"/>
+      <c r="R26" s="116"/>
+      <c r="S26" s="116"/>
+      <c r="T26" s="116"/>
+      <c r="U26" s="116"/>
+      <c r="V26" s="116"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="1"/>
+      <c r="Y26" s="1"/>
+      <c r="Z26" s="1"/>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="1"/>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="1"/>
+      <c r="AH26" s="1"/>
+      <c r="AI26" s="1"/>
+      <c r="AJ26" s="1"/>
+      <c r="AK26" s="1"/>
+      <c r="AL26" s="1"/>
+      <c r="AM26" s="1"/>
+      <c r="AN26" s="1"/>
+    </row>
+    <row r="27" spans="1:40" ht="16.5" customHeight="1">
+      <c r="A27" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="1"/>
-      <c r="R26" s="1"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="1"/>
-      <c r="U26" s="1"/>
-      <c r="V26" s="1"/>
-      <c r="W26" s="73"/>
-      <c r="X26" s="73"/>
-      <c r="Y26" s="73"/>
-      <c r="Z26" s="73"/>
-      <c r="AA26" s="73"/>
-      <c r="AB26" s="1"/>
-      <c r="AC26" s="136"/>
-      <c r="AD26" s="115"/>
-      <c r="AE26" s="115"/>
-      <c r="AF26" s="115"/>
-      <c r="AG26" s="115"/>
-      <c r="AH26" s="115"/>
-      <c r="AI26" s="115"/>
-      <c r="AJ26" s="115"/>
-      <c r="AK26" s="115"/>
-      <c r="AL26" s="115"/>
-      <c r="AM26" s="3"/>
-      <c r="AN26" s="3"/>
-    </row>
-    <row r="27" spans="1:40" ht="14.25" customHeight="1">
-      <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -4066,24 +4144,22 @@
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
-      <c r="W27" s="1"/>
-      <c r="X27" s="1"/>
-      <c r="Y27" s="1"/>
-      <c r="Z27" s="1"/>
-      <c r="AA27" s="1"/>
+      <c r="W27" s="73"/>
+      <c r="X27" s="73"/>
+      <c r="Y27" s="73"/>
+      <c r="Z27" s="73"/>
+      <c r="AA27" s="73"/>
       <c r="AB27" s="1"/>
-      <c r="AC27" s="1"/>
-      <c r="AD27" s="1"/>
-      <c r="AE27" s="1"/>
-      <c r="AF27" s="1"/>
-      <c r="AG27" s="74" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH27" s="3"/>
-      <c r="AI27" s="3"/>
-      <c r="AJ27" s="3"/>
-      <c r="AK27" s="3"/>
-      <c r="AL27" s="3"/>
+      <c r="AC27" s="143"/>
+      <c r="AD27" s="144"/>
+      <c r="AE27" s="144"/>
+      <c r="AF27" s="144"/>
+      <c r="AG27" s="144"/>
+      <c r="AH27" s="144"/>
+      <c r="AI27" s="144"/>
+      <c r="AJ27" s="144"/>
+      <c r="AK27" s="144"/>
+      <c r="AL27" s="144"/>
       <c r="AM27" s="3"/>
       <c r="AN27" s="3"/>
     </row>
@@ -4120,7 +4196,9 @@
       <c r="AD28" s="1"/>
       <c r="AE28" s="1"/>
       <c r="AF28" s="1"/>
-      <c r="AG28" s="74"/>
+      <c r="AG28" s="74" t="s">
+        <v>35</v>
+      </c>
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
       <c r="AJ28" s="3"/>
@@ -4213,29 +4291,29 @@
       <c r="AM30" s="3"/>
       <c r="AN30" s="3"/>
     </row>
-    <row r="31" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A31" s="73"/>
-      <c r="B31" s="73"/>
-      <c r="C31" s="73"/>
-      <c r="D31" s="73"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="73"/>
-      <c r="H31" s="73"/>
-      <c r="I31" s="73"/>
-      <c r="J31" s="73"/>
-      <c r="K31" s="73"/>
-      <c r="L31" s="73"/>
-      <c r="M31" s="73"/>
-      <c r="N31" s="73"/>
-      <c r="O31" s="73"/>
-      <c r="P31" s="73"/>
-      <c r="Q31" s="73"/>
-      <c r="R31" s="73"/>
-      <c r="S31" s="73"/>
-      <c r="T31" s="73"/>
-      <c r="U31" s="73"/>
-      <c r="V31" s="73"/>
+    <row r="31" spans="1:40" ht="14.25" customHeight="1">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
       <c r="W31" s="1"/>
       <c r="X31" s="1"/>
       <c r="Y31" s="1"/>
@@ -4246,48 +4324,42 @@
       <c r="AD31" s="1"/>
       <c r="AE31" s="1"/>
       <c r="AF31" s="1"/>
-      <c r="AG31" s="1"/>
-      <c r="AH31" s="1"/>
-      <c r="AI31" s="1"/>
-      <c r="AJ31" s="1"/>
-      <c r="AK31" s="1"/>
-      <c r="AL31" s="1"/>
-      <c r="AM31" s="1"/>
-      <c r="AN31" s="1"/>
+      <c r="AG31" s="74"/>
+      <c r="AH31" s="3"/>
+      <c r="AI31" s="3"/>
+      <c r="AJ31" s="3"/>
+      <c r="AK31" s="3"/>
+      <c r="AL31" s="3"/>
+      <c r="AM31" s="3"/>
+      <c r="AN31" s="3"/>
     </row>
     <row r="32" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A32" s="75" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="76"/>
-      <c r="C32" s="76"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="111" t="s">
-        <v>37</v>
-      </c>
-      <c r="F32" s="112"/>
-      <c r="G32" s="112"/>
-      <c r="H32" s="112"/>
-      <c r="I32" s="112"/>
-      <c r="J32" s="112"/>
-      <c r="K32" s="112"/>
-      <c r="L32" s="112"/>
-      <c r="M32" s="112"/>
-      <c r="N32" s="112"/>
-      <c r="O32" s="112"/>
-      <c r="P32" s="112"/>
-      <c r="Q32" s="112"/>
-      <c r="R32" s="1"/>
-      <c r="S32" s="1"/>
-      <c r="T32" s="122" t="s">
-        <v>38</v>
-      </c>
-      <c r="U32" s="112"/>
-      <c r="V32" s="112"/>
-      <c r="W32" s="112"/>
-      <c r="X32" s="112"/>
-      <c r="Y32" s="112"/>
-      <c r="Z32" s="112"/>
+      <c r="A32" s="73"/>
+      <c r="B32" s="73"/>
+      <c r="C32" s="73"/>
+      <c r="D32" s="73"/>
+      <c r="E32" s="73"/>
+      <c r="F32" s="73"/>
+      <c r="G32" s="73"/>
+      <c r="H32" s="73"/>
+      <c r="I32" s="73"/>
+      <c r="J32" s="73"/>
+      <c r="K32" s="73"/>
+      <c r="L32" s="73"/>
+      <c r="M32" s="73"/>
+      <c r="N32" s="73"/>
+      <c r="O32" s="73"/>
+      <c r="P32" s="73"/>
+      <c r="Q32" s="73"/>
+      <c r="R32" s="73"/>
+      <c r="S32" s="73"/>
+      <c r="T32" s="73"/>
+      <c r="U32" s="73"/>
+      <c r="V32" s="73"/>
+      <c r="W32" s="1"/>
+      <c r="X32" s="1"/>
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1"/>
       <c r="AA32" s="1"/>
       <c r="AB32" s="1"/>
       <c r="AC32" s="1"/>
@@ -4305,33 +4377,37 @@
     </row>
     <row r="33" spans="1:40" ht="16.5" customHeight="1">
       <c r="A33" s="75" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="77"/>
-      <c r="C33" s="77"/>
+        <v>36</v>
+      </c>
+      <c r="B33" s="76"/>
+      <c r="C33" s="76"/>
       <c r="D33" s="1"/>
-      <c r="E33" s="112"/>
-      <c r="F33" s="112"/>
-      <c r="G33" s="112"/>
-      <c r="H33" s="112"/>
-      <c r="I33" s="112"/>
-      <c r="J33" s="112"/>
-      <c r="K33" s="112"/>
-      <c r="L33" s="112"/>
-      <c r="M33" s="112"/>
-      <c r="N33" s="112"/>
-      <c r="O33" s="112"/>
-      <c r="P33" s="112"/>
-      <c r="Q33" s="112"/>
+      <c r="E33" s="152" t="s">
+        <v>37</v>
+      </c>
+      <c r="F33" s="116"/>
+      <c r="G33" s="116"/>
+      <c r="H33" s="116"/>
+      <c r="I33" s="116"/>
+      <c r="J33" s="116"/>
+      <c r="K33" s="116"/>
+      <c r="L33" s="116"/>
+      <c r="M33" s="116"/>
+      <c r="N33" s="116"/>
+      <c r="O33" s="116"/>
+      <c r="P33" s="116"/>
+      <c r="Q33" s="116"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
-      <c r="T33" s="112"/>
-      <c r="U33" s="112"/>
-      <c r="V33" s="112"/>
-      <c r="W33" s="112"/>
-      <c r="X33" s="112"/>
-      <c r="Y33" s="112"/>
-      <c r="Z33" s="112"/>
+      <c r="T33" s="155" t="s">
+        <v>38</v>
+      </c>
+      <c r="U33" s="116"/>
+      <c r="V33" s="116"/>
+      <c r="W33" s="116"/>
+      <c r="X33" s="116"/>
+      <c r="Y33" s="116"/>
+      <c r="Z33" s="116"/>
       <c r="AA33" s="1"/>
       <c r="AB33" s="1"/>
       <c r="AC33" s="1"/>
@@ -4349,35 +4425,33 @@
     </row>
     <row r="34" spans="1:40" ht="16.5" customHeight="1">
       <c r="A34" s="75" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B34" s="77"/>
       <c r="C34" s="77"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="112"/>
-      <c r="F34" s="112"/>
-      <c r="G34" s="112"/>
-      <c r="H34" s="112"/>
-      <c r="I34" s="112"/>
-      <c r="J34" s="112"/>
-      <c r="K34" s="112"/>
-      <c r="L34" s="112"/>
-      <c r="M34" s="112"/>
-      <c r="N34" s="112"/>
-      <c r="O34" s="112"/>
-      <c r="P34" s="112"/>
-      <c r="Q34" s="112"/>
+      <c r="E34" s="116"/>
+      <c r="F34" s="116"/>
+      <c r="G34" s="116"/>
+      <c r="H34" s="116"/>
+      <c r="I34" s="116"/>
+      <c r="J34" s="116"/>
+      <c r="K34" s="116"/>
+      <c r="L34" s="116"/>
+      <c r="M34" s="116"/>
+      <c r="N34" s="116"/>
+      <c r="O34" s="116"/>
+      <c r="P34" s="116"/>
+      <c r="Q34" s="116"/>
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
-      <c r="T34" s="123" t="s">
-        <v>41</v>
-      </c>
-      <c r="U34" s="112"/>
-      <c r="V34" s="112"/>
-      <c r="W34" s="112"/>
-      <c r="X34" s="112"/>
-      <c r="Y34" s="112"/>
-      <c r="Z34" s="112"/>
+      <c r="T34" s="116"/>
+      <c r="U34" s="116"/>
+      <c r="V34" s="116"/>
+      <c r="W34" s="116"/>
+      <c r="X34" s="116"/>
+      <c r="Y34" s="116"/>
+      <c r="Z34" s="116"/>
       <c r="AA34" s="1"/>
       <c r="AB34" s="1"/>
       <c r="AC34" s="1"/>
@@ -4395,33 +4469,35 @@
     </row>
     <row r="35" spans="1:40" ht="16.5" customHeight="1">
       <c r="A35" s="75" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B35" s="77"/>
       <c r="C35" s="77"/>
       <c r="D35" s="1"/>
-      <c r="E35" s="112"/>
-      <c r="F35" s="112"/>
-      <c r="G35" s="112"/>
-      <c r="H35" s="112"/>
-      <c r="I35" s="112"/>
-      <c r="J35" s="112"/>
-      <c r="K35" s="112"/>
-      <c r="L35" s="112"/>
-      <c r="M35" s="112"/>
-      <c r="N35" s="112"/>
-      <c r="O35" s="112"/>
-      <c r="P35" s="112"/>
-      <c r="Q35" s="112"/>
+      <c r="E35" s="116"/>
+      <c r="F35" s="116"/>
+      <c r="G35" s="116"/>
+      <c r="H35" s="116"/>
+      <c r="I35" s="116"/>
+      <c r="J35" s="116"/>
+      <c r="K35" s="116"/>
+      <c r="L35" s="116"/>
+      <c r="M35" s="116"/>
+      <c r="N35" s="116"/>
+      <c r="O35" s="116"/>
+      <c r="P35" s="116"/>
+      <c r="Q35" s="116"/>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
-      <c r="T35" s="112"/>
-      <c r="U35" s="112"/>
-      <c r="V35" s="112"/>
-      <c r="W35" s="112"/>
-      <c r="X35" s="112"/>
-      <c r="Y35" s="112"/>
-      <c r="Z35" s="112"/>
+      <c r="T35" s="156" t="s">
+        <v>41</v>
+      </c>
+      <c r="U35" s="116"/>
+      <c r="V35" s="116"/>
+      <c r="W35" s="116"/>
+      <c r="X35" s="116"/>
+      <c r="Y35" s="116"/>
+      <c r="Z35" s="116"/>
       <c r="AA35" s="1"/>
       <c r="AB35" s="1"/>
       <c r="AC35" s="1"/>
@@ -4438,32 +4514,34 @@
       <c r="AN35" s="1"/>
     </row>
     <row r="36" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
+      <c r="A36" s="75" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="77"/>
+      <c r="C36" s="77"/>
       <c r="D36" s="1"/>
-      <c r="E36" s="112"/>
-      <c r="F36" s="112"/>
-      <c r="G36" s="112"/>
-      <c r="H36" s="112"/>
-      <c r="I36" s="112"/>
-      <c r="J36" s="112"/>
-      <c r="K36" s="112"/>
-      <c r="L36" s="112"/>
-      <c r="M36" s="112"/>
-      <c r="N36" s="112"/>
-      <c r="O36" s="112"/>
-      <c r="P36" s="112"/>
-      <c r="Q36" s="112"/>
+      <c r="E36" s="116"/>
+      <c r="F36" s="116"/>
+      <c r="G36" s="116"/>
+      <c r="H36" s="116"/>
+      <c r="I36" s="116"/>
+      <c r="J36" s="116"/>
+      <c r="K36" s="116"/>
+      <c r="L36" s="116"/>
+      <c r="M36" s="116"/>
+      <c r="N36" s="116"/>
+      <c r="O36" s="116"/>
+      <c r="P36" s="116"/>
+      <c r="Q36" s="116"/>
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
-      <c r="T36" s="1"/>
-      <c r="U36" s="1"/>
-      <c r="V36" s="1"/>
-      <c r="W36" s="1"/>
-      <c r="X36" s="1"/>
-      <c r="Y36" s="1"/>
-      <c r="Z36" s="1"/>
+      <c r="T36" s="116"/>
+      <c r="U36" s="116"/>
+      <c r="V36" s="116"/>
+      <c r="W36" s="116"/>
+      <c r="X36" s="116"/>
+      <c r="Y36" s="116"/>
+      <c r="Z36" s="116"/>
       <c r="AA36" s="1"/>
       <c r="AB36" s="1"/>
       <c r="AC36" s="1"/>
@@ -4484,19 +4562,19 @@
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
-      <c r="E37" s="112"/>
-      <c r="F37" s="112"/>
-      <c r="G37" s="112"/>
-      <c r="H37" s="112"/>
-      <c r="I37" s="112"/>
-      <c r="J37" s="112"/>
-      <c r="K37" s="112"/>
-      <c r="L37" s="112"/>
-      <c r="M37" s="112"/>
-      <c r="N37" s="112"/>
-      <c r="O37" s="112"/>
-      <c r="P37" s="112"/>
-      <c r="Q37" s="112"/>
+      <c r="E37" s="116"/>
+      <c r="F37" s="116"/>
+      <c r="G37" s="116"/>
+      <c r="H37" s="116"/>
+      <c r="I37" s="116"/>
+      <c r="J37" s="116"/>
+      <c r="K37" s="116"/>
+      <c r="L37" s="116"/>
+      <c r="M37" s="116"/>
+      <c r="N37" s="116"/>
+      <c r="O37" s="116"/>
+      <c r="P37" s="116"/>
+      <c r="Q37" s="116"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
@@ -4526,19 +4604,19 @@
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-      <c r="P38" s="1"/>
-      <c r="Q38" s="1"/>
+      <c r="E38" s="116"/>
+      <c r="F38" s="116"/>
+      <c r="G38" s="116"/>
+      <c r="H38" s="116"/>
+      <c r="I38" s="116"/>
+      <c r="J38" s="116"/>
+      <c r="K38" s="116"/>
+      <c r="L38" s="116"/>
+      <c r="M38" s="116"/>
+      <c r="N38" s="116"/>
+      <c r="O38" s="116"/>
+      <c r="P38" s="116"/>
+      <c r="Q38" s="116"/>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
       <c r="T38" s="1"/>
@@ -12837,8 +12915,94 @@
       <c r="AM235" s="1"/>
       <c r="AN235" s="1"/>
     </row>
+    <row r="236" spans="1:40" ht="16.5" customHeight="1">
+      <c r="A236" s="1"/>
+      <c r="B236" s="1"/>
+      <c r="C236" s="1"/>
+      <c r="D236" s="1"/>
+      <c r="E236" s="1"/>
+      <c r="F236" s="1"/>
+      <c r="G236" s="1"/>
+      <c r="H236" s="1"/>
+      <c r="I236" s="1"/>
+      <c r="J236" s="1"/>
+      <c r="K236" s="1"/>
+      <c r="L236" s="1"/>
+      <c r="M236" s="1"/>
+      <c r="N236" s="1"/>
+      <c r="O236" s="1"/>
+      <c r="P236" s="1"/>
+      <c r="Q236" s="1"/>
+      <c r="R236" s="1"/>
+      <c r="S236" s="1"/>
+      <c r="T236" s="1"/>
+      <c r="U236" s="1"/>
+      <c r="V236" s="1"/>
+      <c r="W236" s="1"/>
+      <c r="X236" s="1"/>
+      <c r="Y236" s="1"/>
+      <c r="Z236" s="1"/>
+      <c r="AA236" s="1"/>
+      <c r="AB236" s="1"/>
+      <c r="AC236" s="1"/>
+      <c r="AD236" s="1"/>
+      <c r="AE236" s="1"/>
+      <c r="AF236" s="1"/>
+      <c r="AG236" s="1"/>
+      <c r="AH236" s="1"/>
+      <c r="AI236" s="1"/>
+      <c r="AJ236" s="1"/>
+      <c r="AK236" s="1"/>
+      <c r="AL236" s="1"/>
+      <c r="AM236" s="1"/>
+      <c r="AN236" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="52">
+  <mergeCells count="53">
+    <mergeCell ref="E33:Q38"/>
+    <mergeCell ref="A26:V26"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="T10:V10"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="Q10:S10"/>
+    <mergeCell ref="T33:Z34"/>
+    <mergeCell ref="T35:Z36"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="E9:G10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="AC27:AL27"/>
+    <mergeCell ref="H9:M9"/>
+    <mergeCell ref="W9:AE9"/>
+    <mergeCell ref="N9:V9"/>
+    <mergeCell ref="AL10:AN10"/>
+    <mergeCell ref="Z10:AB10"/>
+    <mergeCell ref="AC10:AE10"/>
+    <mergeCell ref="AF10:AH10"/>
+    <mergeCell ref="AI10:AK10"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="C9:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C7:P7"/>
+    <mergeCell ref="U7:X7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="E19:AN19"/>
+    <mergeCell ref="Y7:AC7"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="AE7:AI7"/>
+    <mergeCell ref="AF9:AN9"/>
+    <mergeCell ref="AJ7:AN7"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="C18:D18"/>
     <mergeCell ref="N5:U5"/>
     <mergeCell ref="A1:AN2"/>
     <mergeCell ref="A3:AN3"/>
@@ -12848,49 +13012,6 @@
     <mergeCell ref="Y5:AF5"/>
     <mergeCell ref="W5:X5"/>
     <mergeCell ref="L5:M5"/>
-    <mergeCell ref="C7:P7"/>
-    <mergeCell ref="U7:X7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="E18:AN18"/>
-    <mergeCell ref="Y7:AC7"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="AE7:AI7"/>
-    <mergeCell ref="AF9:AN9"/>
-    <mergeCell ref="AJ7:AN7"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="C9:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="AC26:AL26"/>
-    <mergeCell ref="H9:M9"/>
-    <mergeCell ref="W9:AE9"/>
-    <mergeCell ref="N9:V9"/>
-    <mergeCell ref="AL10:AN10"/>
-    <mergeCell ref="Z10:AB10"/>
-    <mergeCell ref="AC10:AE10"/>
-    <mergeCell ref="AF10:AH10"/>
-    <mergeCell ref="AI10:AK10"/>
-    <mergeCell ref="E32:Q37"/>
-    <mergeCell ref="A25:V25"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="T10:V10"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="T32:Z33"/>
-    <mergeCell ref="T34:Z35"/>
-    <mergeCell ref="W10:Y10"/>
-    <mergeCell ref="E9:G10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A22:D22"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.17" right="0.16" top="0.23" bottom="0.19" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat(admin): update admin dashboard and fix SF4 exports
add real-time clock and redesigned last scanned learner card on admin dashboard
fix SF4 template row count and indentation in SF4_MAPPINGS
add custom JHS section sorting order for SF4 exports
add debug logging for SF4 adviser mappings
remove unnecessary not-null filter for section_assigned in export queries
update profile handling to support section_assigned field
update admin login page to include section_assigned in profile data
</commit_message>
<xml_diff>
--- a/assets/admin/attendance/templates/SF4_Blank.xlsx
+++ b/assets/admin/attendance/templates/SF4_Blank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\L4T\Documents\Website\ulhs.github.io\assets\admin\attendance\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F409E2-9757-4606-A183-27CD87CAC7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D61891FC-1D99-4F25-B963-BF2A0FEAAB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1595,6 +1595,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1709,18 +1721,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1987,141 +1987,142 @@
     <col min="3" max="3" width="11.7265625" customWidth="1"/>
     <col min="4" max="4" width="16.26953125" customWidth="1"/>
     <col min="5" max="7" width="4.7265625" customWidth="1"/>
-    <col min="8" max="9" width="5.7265625" customWidth="1"/>
-    <col min="10" max="10" width="6.54296875" customWidth="1"/>
-    <col min="11" max="13" width="5.7265625" customWidth="1"/>
+    <col min="8" max="9" width="5.90625" customWidth="1"/>
+    <col min="10" max="10" width="7.26953125" customWidth="1"/>
+    <col min="11" max="12" width="5.90625" customWidth="1"/>
+    <col min="13" max="13" width="7.26953125" customWidth="1"/>
     <col min="14" max="40" width="3.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A1" s="115" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
-      <c r="AD1" s="116"/>
-      <c r="AE1" s="116"/>
-      <c r="AF1" s="116"/>
-      <c r="AG1" s="116"/>
-      <c r="AH1" s="116"/>
-      <c r="AI1" s="116"/>
-      <c r="AJ1" s="116"/>
-      <c r="AK1" s="116"/>
-      <c r="AL1" s="116"/>
-      <c r="AM1" s="116"/>
-      <c r="AN1" s="116"/>
+      <c r="A1" s="119" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="120"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
+      <c r="F1" s="120"/>
+      <c r="G1" s="120"/>
+      <c r="H1" s="120"/>
+      <c r="I1" s="120"/>
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="120"/>
+      <c r="T1" s="120"/>
+      <c r="U1" s="120"/>
+      <c r="V1" s="120"/>
+      <c r="W1" s="120"/>
+      <c r="X1" s="120"/>
+      <c r="Y1" s="120"/>
+      <c r="Z1" s="120"/>
+      <c r="AA1" s="120"/>
+      <c r="AB1" s="120"/>
+      <c r="AC1" s="120"/>
+      <c r="AD1" s="120"/>
+      <c r="AE1" s="120"/>
+      <c r="AF1" s="120"/>
+      <c r="AG1" s="120"/>
+      <c r="AH1" s="120"/>
+      <c r="AI1" s="120"/>
+      <c r="AJ1" s="120"/>
+      <c r="AK1" s="120"/>
+      <c r="AL1" s="120"/>
+      <c r="AM1" s="120"/>
+      <c r="AN1" s="120"/>
     </row>
     <row r="2" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A2" s="116"/>
-      <c r="B2" s="116"/>
-      <c r="C2" s="116"/>
-      <c r="D2" s="116"/>
-      <c r="E2" s="116"/>
-      <c r="F2" s="116"/>
-      <c r="G2" s="116"/>
-      <c r="H2" s="116"/>
-      <c r="I2" s="116"/>
-      <c r="J2" s="116"/>
-      <c r="K2" s="116"/>
-      <c r="L2" s="116"/>
-      <c r="M2" s="116"/>
-      <c r="N2" s="116"/>
-      <c r="O2" s="116"/>
-      <c r="P2" s="116"/>
-      <c r="Q2" s="116"/>
-      <c r="R2" s="116"/>
-      <c r="S2" s="116"/>
-      <c r="T2" s="116"/>
-      <c r="U2" s="116"/>
-      <c r="V2" s="116"/>
-      <c r="W2" s="116"/>
-      <c r="X2" s="116"/>
-      <c r="Y2" s="116"/>
-      <c r="Z2" s="116"/>
-      <c r="AA2" s="116"/>
-      <c r="AB2" s="116"/>
-      <c r="AC2" s="116"/>
-      <c r="AD2" s="116"/>
-      <c r="AE2" s="116"/>
-      <c r="AF2" s="116"/>
-      <c r="AG2" s="116"/>
-      <c r="AH2" s="116"/>
-      <c r="AI2" s="116"/>
-      <c r="AJ2" s="116"/>
-      <c r="AK2" s="116"/>
-      <c r="AL2" s="116"/>
-      <c r="AM2" s="116"/>
-      <c r="AN2" s="116"/>
+      <c r="A2" s="120"/>
+      <c r="B2" s="120"/>
+      <c r="C2" s="120"/>
+      <c r="D2" s="120"/>
+      <c r="E2" s="120"/>
+      <c r="F2" s="120"/>
+      <c r="G2" s="120"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="120"/>
+      <c r="J2" s="120"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="120"/>
+      <c r="M2" s="120"/>
+      <c r="N2" s="120"/>
+      <c r="O2" s="120"/>
+      <c r="P2" s="120"/>
+      <c r="Q2" s="120"/>
+      <c r="R2" s="120"/>
+      <c r="S2" s="120"/>
+      <c r="T2" s="120"/>
+      <c r="U2" s="120"/>
+      <c r="V2" s="120"/>
+      <c r="W2" s="120"/>
+      <c r="X2" s="120"/>
+      <c r="Y2" s="120"/>
+      <c r="Z2" s="120"/>
+      <c r="AA2" s="120"/>
+      <c r="AB2" s="120"/>
+      <c r="AC2" s="120"/>
+      <c r="AD2" s="120"/>
+      <c r="AE2" s="120"/>
+      <c r="AF2" s="120"/>
+      <c r="AG2" s="120"/>
+      <c r="AH2" s="120"/>
+      <c r="AI2" s="120"/>
+      <c r="AJ2" s="120"/>
+      <c r="AK2" s="120"/>
+      <c r="AL2" s="120"/>
+      <c r="AM2" s="120"/>
+      <c r="AN2" s="120"/>
     </row>
     <row r="3" spans="1:40" ht="27" customHeight="1">
-      <c r="A3" s="117" t="s">
+      <c r="A3" s="121" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="116"/>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="116"/>
-      <c r="M3" s="116"/>
-      <c r="N3" s="116"/>
-      <c r="O3" s="116"/>
-      <c r="P3" s="116"/>
-      <c r="Q3" s="116"/>
-      <c r="R3" s="116"/>
-      <c r="S3" s="116"/>
-      <c r="T3" s="116"/>
-      <c r="U3" s="116"/>
-      <c r="V3" s="116"/>
-      <c r="W3" s="116"/>
-      <c r="X3" s="116"/>
-      <c r="Y3" s="116"/>
-      <c r="Z3" s="116"/>
-      <c r="AA3" s="116"/>
-      <c r="AB3" s="116"/>
-      <c r="AC3" s="116"/>
-      <c r="AD3" s="116"/>
-      <c r="AE3" s="116"/>
-      <c r="AF3" s="116"/>
-      <c r="AG3" s="116"/>
-      <c r="AH3" s="116"/>
-      <c r="AI3" s="116"/>
-      <c r="AJ3" s="116"/>
-      <c r="AK3" s="116"/>
-      <c r="AL3" s="116"/>
-      <c r="AM3" s="116"/>
-      <c r="AN3" s="116"/>
+      <c r="B3" s="120"/>
+      <c r="C3" s="120"/>
+      <c r="D3" s="120"/>
+      <c r="E3" s="120"/>
+      <c r="F3" s="120"/>
+      <c r="G3" s="120"/>
+      <c r="H3" s="120"/>
+      <c r="I3" s="120"/>
+      <c r="J3" s="120"/>
+      <c r="K3" s="120"/>
+      <c r="L3" s="120"/>
+      <c r="M3" s="120"/>
+      <c r="N3" s="120"/>
+      <c r="O3" s="120"/>
+      <c r="P3" s="120"/>
+      <c r="Q3" s="120"/>
+      <c r="R3" s="120"/>
+      <c r="S3" s="120"/>
+      <c r="T3" s="120"/>
+      <c r="U3" s="120"/>
+      <c r="V3" s="120"/>
+      <c r="W3" s="120"/>
+      <c r="X3" s="120"/>
+      <c r="Y3" s="120"/>
+      <c r="Z3" s="120"/>
+      <c r="AA3" s="120"/>
+      <c r="AB3" s="120"/>
+      <c r="AC3" s="120"/>
+      <c r="AD3" s="120"/>
+      <c r="AE3" s="120"/>
+      <c r="AF3" s="120"/>
+      <c r="AG3" s="120"/>
+      <c r="AH3" s="120"/>
+      <c r="AI3" s="120"/>
+      <c r="AJ3" s="120"/>
+      <c r="AK3" s="120"/>
+      <c r="AL3" s="120"/>
+      <c r="AM3" s="120"/>
+      <c r="AN3" s="120"/>
     </row>
     <row r="4" spans="1:40" ht="20.25" customHeight="1">
       <c r="A4" s="1"/>
@@ -2171,41 +2172,41 @@
       <c r="C5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="112"/>
-      <c r="E5" s="113"/>
-      <c r="F5" s="114"/>
-      <c r="G5" s="118" t="s">
+      <c r="D5" s="116"/>
+      <c r="E5" s="117"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="122" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="119"/>
-      <c r="I5" s="112"/>
-      <c r="J5" s="114"/>
+      <c r="H5" s="123"/>
+      <c r="I5" s="116"/>
+      <c r="J5" s="118"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="118" t="s">
+      <c r="L5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="119"/>
-      <c r="N5" s="112"/>
-      <c r="O5" s="113"/>
-      <c r="P5" s="113"/>
-      <c r="Q5" s="113"/>
-      <c r="R5" s="113"/>
-      <c r="S5" s="113"/>
-      <c r="T5" s="113"/>
-      <c r="U5" s="114"/>
+      <c r="M5" s="123"/>
+      <c r="N5" s="116"/>
+      <c r="O5" s="117"/>
+      <c r="P5" s="117"/>
+      <c r="Q5" s="117"/>
+      <c r="R5" s="117"/>
+      <c r="S5" s="117"/>
+      <c r="T5" s="117"/>
+      <c r="U5" s="118"/>
       <c r="V5" s="2"/>
-      <c r="W5" s="118" t="s">
+      <c r="W5" s="122" t="s">
         <v>5</v>
       </c>
-      <c r="X5" s="119"/>
-      <c r="Y5" s="112"/>
-      <c r="Z5" s="113"/>
-      <c r="AA5" s="113"/>
-      <c r="AB5" s="113"/>
-      <c r="AC5" s="113"/>
-      <c r="AD5" s="113"/>
-      <c r="AE5" s="113"/>
-      <c r="AF5" s="114"/>
+      <c r="X5" s="123"/>
+      <c r="Y5" s="116"/>
+      <c r="Z5" s="117"/>
+      <c r="AA5" s="117"/>
+      <c r="AB5" s="117"/>
+      <c r="AC5" s="117"/>
+      <c r="AD5" s="117"/>
+      <c r="AE5" s="117"/>
+      <c r="AF5" s="118"/>
       <c r="AG5" s="5"/>
       <c r="AH5" s="5"/>
       <c r="AI5" s="5"/>
@@ -2258,52 +2259,52 @@
       <c r="AN6" s="5"/>
     </row>
     <row r="7" spans="1:40" ht="26.25" customHeight="1">
-      <c r="A7" s="118" t="s">
+      <c r="A7" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="119"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
-      <c r="H7" s="113"/>
-      <c r="I7" s="113"/>
-      <c r="J7" s="113"/>
-      <c r="K7" s="113"/>
-      <c r="L7" s="113"/>
-      <c r="M7" s="113"/>
-      <c r="N7" s="113"/>
-      <c r="O7" s="113"/>
-      <c r="P7" s="114"/>
+      <c r="B7" s="123"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="117"/>
+      <c r="E7" s="117"/>
+      <c r="F7" s="117"/>
+      <c r="G7" s="117"/>
+      <c r="H7" s="117"/>
+      <c r="I7" s="117"/>
+      <c r="J7" s="117"/>
+      <c r="K7" s="117"/>
+      <c r="L7" s="117"/>
+      <c r="M7" s="117"/>
+      <c r="N7" s="117"/>
+      <c r="O7" s="117"/>
+      <c r="P7" s="118"/>
       <c r="Q7" s="5"/>
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
       <c r="T7" s="5"/>
-      <c r="U7" s="118" t="s">
+      <c r="U7" s="122" t="s">
         <v>7</v>
       </c>
-      <c r="V7" s="116"/>
-      <c r="W7" s="116"/>
-      <c r="X7" s="119"/>
-      <c r="Y7" s="112"/>
-      <c r="Z7" s="113"/>
-      <c r="AA7" s="113"/>
-      <c r="AB7" s="113"/>
-      <c r="AC7" s="114"/>
+      <c r="V7" s="120"/>
+      <c r="W7" s="120"/>
+      <c r="X7" s="123"/>
+      <c r="Y7" s="116"/>
+      <c r="Z7" s="117"/>
+      <c r="AA7" s="117"/>
+      <c r="AB7" s="117"/>
+      <c r="AC7" s="118"/>
       <c r="AD7" s="5"/>
-      <c r="AE7" s="129" t="s">
+      <c r="AE7" s="133" t="s">
         <v>8</v>
       </c>
-      <c r="AF7" s="116"/>
-      <c r="AG7" s="116"/>
-      <c r="AH7" s="116"/>
-      <c r="AI7" s="119"/>
-      <c r="AJ7" s="112"/>
-      <c r="AK7" s="113"/>
-      <c r="AL7" s="113"/>
-      <c r="AM7" s="113"/>
-      <c r="AN7" s="114"/>
+      <c r="AF7" s="120"/>
+      <c r="AG7" s="120"/>
+      <c r="AH7" s="120"/>
+      <c r="AI7" s="123"/>
+      <c r="AJ7" s="116"/>
+      <c r="AK7" s="117"/>
+      <c r="AL7" s="117"/>
+      <c r="AM7" s="117"/>
+      <c r="AN7" s="118"/>
     </row>
     <row r="8" spans="1:40" ht="6.75" customHeight="1">
       <c r="A8" s="1"/>
@@ -2348,132 +2349,132 @@
       <c r="AN8" s="1"/>
     </row>
     <row r="9" spans="1:40" ht="21" customHeight="1">
-      <c r="A9" s="120" t="s">
+      <c r="A9" s="124" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="133" t="s">
+      <c r="B9" s="137" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="133" t="s">
+      <c r="C9" s="137" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="139"/>
-      <c r="E9" s="133" t="s">
+      <c r="D9" s="143"/>
+      <c r="E9" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="139"/>
-      <c r="G9" s="157"/>
-      <c r="H9" s="145" t="s">
+      <c r="F9" s="143"/>
+      <c r="G9" s="161"/>
+      <c r="H9" s="149" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="127"/>
-      <c r="J9" s="127"/>
-      <c r="K9" s="127"/>
-      <c r="L9" s="127"/>
-      <c r="M9" s="127"/>
-      <c r="N9" s="130" t="s">
+      <c r="I9" s="131"/>
+      <c r="J9" s="131"/>
+      <c r="K9" s="131"/>
+      <c r="L9" s="131"/>
+      <c r="M9" s="131"/>
+      <c r="N9" s="134" t="s">
         <v>14</v>
       </c>
-      <c r="O9" s="127"/>
-      <c r="P9" s="127"/>
-      <c r="Q9" s="127"/>
-      <c r="R9" s="127"/>
-      <c r="S9" s="127"/>
-      <c r="T9" s="127"/>
-      <c r="U9" s="127"/>
-      <c r="V9" s="128"/>
-      <c r="W9" s="145" t="s">
+      <c r="O9" s="131"/>
+      <c r="P9" s="131"/>
+      <c r="Q9" s="131"/>
+      <c r="R9" s="131"/>
+      <c r="S9" s="131"/>
+      <c r="T9" s="131"/>
+      <c r="U9" s="131"/>
+      <c r="V9" s="132"/>
+      <c r="W9" s="149" t="s">
         <v>15</v>
       </c>
-      <c r="X9" s="127"/>
-      <c r="Y9" s="127"/>
-      <c r="Z9" s="127"/>
-      <c r="AA9" s="127"/>
-      <c r="AB9" s="127"/>
-      <c r="AC9" s="127"/>
-      <c r="AD9" s="127"/>
-      <c r="AE9" s="127"/>
-      <c r="AF9" s="130" t="s">
+      <c r="X9" s="131"/>
+      <c r="Y9" s="131"/>
+      <c r="Z9" s="131"/>
+      <c r="AA9" s="131"/>
+      <c r="AB9" s="131"/>
+      <c r="AC9" s="131"/>
+      <c r="AD9" s="131"/>
+      <c r="AE9" s="131"/>
+      <c r="AF9" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="AG9" s="127"/>
-      <c r="AH9" s="127"/>
-      <c r="AI9" s="127"/>
-      <c r="AJ9" s="127"/>
-      <c r="AK9" s="127"/>
-      <c r="AL9" s="127"/>
-      <c r="AM9" s="127"/>
-      <c r="AN9" s="128"/>
+      <c r="AG9" s="131"/>
+      <c r="AH9" s="131"/>
+      <c r="AI9" s="131"/>
+      <c r="AJ9" s="131"/>
+      <c r="AK9" s="131"/>
+      <c r="AL9" s="131"/>
+      <c r="AM9" s="131"/>
+      <c r="AN9" s="132"/>
     </row>
     <row r="10" spans="1:40" ht="60.75" customHeight="1">
-      <c r="A10" s="121"/>
-      <c r="B10" s="134"/>
-      <c r="C10" s="134"/>
-      <c r="D10" s="116"/>
-      <c r="E10" s="134"/>
-      <c r="F10" s="116"/>
-      <c r="G10" s="158"/>
-      <c r="H10" s="159" t="s">
+      <c r="A10" s="125"/>
+      <c r="B10" s="138"/>
+      <c r="C10" s="138"/>
+      <c r="D10" s="120"/>
+      <c r="E10" s="138"/>
+      <c r="F10" s="120"/>
+      <c r="G10" s="162"/>
+      <c r="H10" s="163" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="147"/>
-      <c r="J10" s="149"/>
-      <c r="K10" s="154" t="s">
+      <c r="I10" s="151"/>
+      <c r="J10" s="153"/>
+      <c r="K10" s="158" t="s">
         <v>18</v>
       </c>
-      <c r="L10" s="144"/>
-      <c r="M10" s="151"/>
-      <c r="N10" s="150" t="s">
+      <c r="L10" s="148"/>
+      <c r="M10" s="155"/>
+      <c r="N10" s="154" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="144"/>
-      <c r="P10" s="151"/>
-      <c r="Q10" s="146" t="s">
+      <c r="O10" s="148"/>
+      <c r="P10" s="155"/>
+      <c r="Q10" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="R10" s="147"/>
-      <c r="S10" s="149"/>
-      <c r="T10" s="146" t="s">
+      <c r="R10" s="151"/>
+      <c r="S10" s="153"/>
+      <c r="T10" s="150" t="s">
         <v>21</v>
       </c>
-      <c r="U10" s="147"/>
-      <c r="V10" s="148"/>
-      <c r="W10" s="150" t="s">
+      <c r="U10" s="151"/>
+      <c r="V10" s="152"/>
+      <c r="W10" s="154" t="s">
         <v>19</v>
       </c>
-      <c r="X10" s="144"/>
-      <c r="Y10" s="151"/>
-      <c r="Z10" s="146" t="s">
+      <c r="X10" s="148"/>
+      <c r="Y10" s="155"/>
+      <c r="Z10" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="AA10" s="147"/>
-      <c r="AB10" s="149"/>
-      <c r="AC10" s="146" t="s">
+      <c r="AA10" s="151"/>
+      <c r="AB10" s="153"/>
+      <c r="AC10" s="150" t="s">
         <v>21</v>
       </c>
-      <c r="AD10" s="147"/>
-      <c r="AE10" s="148"/>
-      <c r="AF10" s="150" t="s">
+      <c r="AD10" s="151"/>
+      <c r="AE10" s="152"/>
+      <c r="AF10" s="154" t="s">
         <v>19</v>
       </c>
-      <c r="AG10" s="144"/>
-      <c r="AH10" s="151"/>
-      <c r="AI10" s="146" t="s">
+      <c r="AG10" s="148"/>
+      <c r="AH10" s="155"/>
+      <c r="AI10" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="AJ10" s="147"/>
-      <c r="AK10" s="149"/>
-      <c r="AL10" s="146" t="s">
+      <c r="AJ10" s="151"/>
+      <c r="AK10" s="153"/>
+      <c r="AL10" s="150" t="s">
         <v>21</v>
       </c>
-      <c r="AM10" s="147"/>
-      <c r="AN10" s="148"/>
+      <c r="AM10" s="151"/>
+      <c r="AN10" s="152"/>
     </row>
     <row r="11" spans="1:40" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A11" s="122"/>
-      <c r="B11" s="135"/>
-      <c r="C11" s="135"/>
-      <c r="D11" s="124"/>
+      <c r="A11" s="126"/>
+      <c r="B11" s="139"/>
+      <c r="C11" s="139"/>
+      <c r="D11" s="128"/>
       <c r="E11" s="7" t="s">
         <v>22</v>
       </c>
@@ -2588,13 +2589,17 @@
         <v>25</v>
       </c>
       <c r="B12" s="12"/>
-      <c r="C12" s="140"/>
-      <c r="D12" s="141"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="14"/>
+      <c r="C12" s="144"/>
+      <c r="D12" s="145"/>
+      <c r="E12" s="13">
+        <v>1</v>
+      </c>
+      <c r="F12" s="14">
+        <v>2</v>
+      </c>
       <c r="G12" s="15">
         <f t="shared" ref="G12:G18" si="0">SUM(E12:F12)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H12" s="16"/>
       <c r="I12" s="17"/>
@@ -2695,13 +2700,17 @@
         <v>25</v>
       </c>
       <c r="B13" s="82"/>
-      <c r="C13" s="163"/>
-      <c r="D13" s="164"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="84"/>
+      <c r="C13" s="167"/>
+      <c r="D13" s="168"/>
+      <c r="E13" s="83">
+        <v>1</v>
+      </c>
+      <c r="F13" s="84">
+        <v>2</v>
+      </c>
       <c r="G13" s="85">
         <f t="shared" ref="G13:G14" si="3">SUM(E13:F13)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H13" s="79"/>
       <c r="I13" s="80"/>
@@ -2802,13 +2811,17 @@
         <v>26</v>
       </c>
       <c r="B14" s="23"/>
-      <c r="C14" s="131"/>
-      <c r="D14" s="132"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="25"/>
+      <c r="C14" s="135"/>
+      <c r="D14" s="136"/>
+      <c r="E14" s="24">
+        <v>3</v>
+      </c>
+      <c r="F14" s="25">
+        <v>2</v>
+      </c>
       <c r="G14" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H14" s="79"/>
       <c r="I14" s="80"/>
@@ -2909,13 +2922,17 @@
         <v>26</v>
       </c>
       <c r="B15" s="23"/>
-      <c r="C15" s="131"/>
-      <c r="D15" s="132"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="25"/>
+      <c r="C15" s="135"/>
+      <c r="D15" s="136"/>
+      <c r="E15" s="24">
+        <v>2</v>
+      </c>
+      <c r="F15" s="25">
+        <v>3</v>
+      </c>
       <c r="G15" s="26">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H15" s="27"/>
       <c r="I15" s="28"/>
@@ -3016,13 +3033,17 @@
         <v>27</v>
       </c>
       <c r="B16" s="34"/>
-      <c r="C16" s="142"/>
-      <c r="D16" s="132"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="36"/>
+      <c r="C16" s="146"/>
+      <c r="D16" s="136"/>
+      <c r="E16" s="35">
+        <v>1</v>
+      </c>
+      <c r="F16" s="36">
+        <v>1</v>
+      </c>
       <c r="G16" s="37">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H16" s="27"/>
       <c r="I16" s="28"/>
@@ -3123,22 +3144,26 @@
         <v>27</v>
       </c>
       <c r="B17" s="34"/>
-      <c r="C17" s="142"/>
-      <c r="D17" s="132"/>
-      <c r="E17" s="167"/>
-      <c r="F17" s="168"/>
+      <c r="C17" s="146"/>
+      <c r="D17" s="136"/>
+      <c r="E17" s="112">
+        <v>1</v>
+      </c>
+      <c r="F17" s="113">
+        <v>1</v>
+      </c>
       <c r="G17" s="37">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H17" s="169"/>
-      <c r="I17" s="170"/>
+        <v>2</v>
+      </c>
+      <c r="H17" s="114"/>
+      <c r="I17" s="115"/>
       <c r="J17" s="28">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K17" s="170"/>
-      <c r="L17" s="170"/>
+      <c r="K17" s="115"/>
+      <c r="L17" s="115"/>
       <c r="M17" s="88" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
@@ -3230,13 +3255,17 @@
         <v>28</v>
       </c>
       <c r="B18" s="39"/>
-      <c r="C18" s="136"/>
-      <c r="D18" s="132"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="41"/>
+      <c r="C18" s="140"/>
+      <c r="D18" s="136"/>
+      <c r="E18" s="40">
+        <v>2</v>
+      </c>
+      <c r="F18" s="41">
+        <v>2</v>
+      </c>
       <c r="G18" s="42">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18" s="43"/>
       <c r="I18" s="44"/>
@@ -3333,68 +3362,68 @@
       </c>
     </row>
     <row r="19" spans="1:40" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A19" s="126" t="s">
+      <c r="A19" s="130" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="127"/>
-      <c r="C19" s="127"/>
-      <c r="D19" s="128"/>
-      <c r="E19" s="123"/>
-      <c r="F19" s="124"/>
-      <c r="G19" s="124"/>
-      <c r="H19" s="124"/>
-      <c r="I19" s="124"/>
-      <c r="J19" s="124"/>
-      <c r="K19" s="124"/>
-      <c r="L19" s="124"/>
-      <c r="M19" s="124"/>
-      <c r="N19" s="124"/>
-      <c r="O19" s="124"/>
-      <c r="P19" s="124"/>
-      <c r="Q19" s="124"/>
-      <c r="R19" s="124"/>
-      <c r="S19" s="124"/>
-      <c r="T19" s="124"/>
-      <c r="U19" s="124"/>
-      <c r="V19" s="124"/>
-      <c r="W19" s="124"/>
-      <c r="X19" s="124"/>
-      <c r="Y19" s="124"/>
-      <c r="Z19" s="124"/>
-      <c r="AA19" s="124"/>
-      <c r="AB19" s="124"/>
-      <c r="AC19" s="124"/>
-      <c r="AD19" s="124"/>
-      <c r="AE19" s="124"/>
-      <c r="AF19" s="124"/>
-      <c r="AG19" s="124"/>
-      <c r="AH19" s="124"/>
-      <c r="AI19" s="124"/>
-      <c r="AJ19" s="124"/>
-      <c r="AK19" s="124"/>
-      <c r="AL19" s="124"/>
-      <c r="AM19" s="124"/>
-      <c r="AN19" s="125"/>
+      <c r="B19" s="131"/>
+      <c r="C19" s="131"/>
+      <c r="D19" s="132"/>
+      <c r="E19" s="127"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
+      <c r="H19" s="128"/>
+      <c r="I19" s="128"/>
+      <c r="J19" s="128"/>
+      <c r="K19" s="128"/>
+      <c r="L19" s="128"/>
+      <c r="M19" s="128"/>
+      <c r="N19" s="128"/>
+      <c r="O19" s="128"/>
+      <c r="P19" s="128"/>
+      <c r="Q19" s="128"/>
+      <c r="R19" s="128"/>
+      <c r="S19" s="128"/>
+      <c r="T19" s="128"/>
+      <c r="U19" s="128"/>
+      <c r="V19" s="128"/>
+      <c r="W19" s="128"/>
+      <c r="X19" s="128"/>
+      <c r="Y19" s="128"/>
+      <c r="Z19" s="128"/>
+      <c r="AA19" s="128"/>
+      <c r="AB19" s="128"/>
+      <c r="AC19" s="128"/>
+      <c r="AD19" s="128"/>
+      <c r="AE19" s="128"/>
+      <c r="AF19" s="128"/>
+      <c r="AG19" s="128"/>
+      <c r="AH19" s="128"/>
+      <c r="AI19" s="128"/>
+      <c r="AJ19" s="128"/>
+      <c r="AK19" s="128"/>
+      <c r="AL19" s="128"/>
+      <c r="AM19" s="128"/>
+      <c r="AN19" s="129"/>
     </row>
     <row r="20" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A20" s="160" t="str">
+      <c r="A20" s="164" t="str">
         <f>A12</f>
         <v>Grade 7 (I)</v>
       </c>
-      <c r="B20" s="161"/>
-      <c r="C20" s="161"/>
-      <c r="D20" s="161"/>
+      <c r="B20" s="165"/>
+      <c r="C20" s="165"/>
+      <c r="D20" s="165"/>
       <c r="E20" s="45">
         <f>SUM(E12:E13)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" s="46">
         <f>SUM(F12:F13)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G20" s="47">
         <f>SUM(E20:F20)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H20" s="48">
         <f>SUM(H12:H13)</f>
@@ -3503,23 +3532,23 @@
       </c>
     </row>
     <row r="21" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A21" s="162" t="s">
+      <c r="A21" s="166" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="113"/>
-      <c r="C21" s="113"/>
-      <c r="D21" s="113"/>
+      <c r="B21" s="117"/>
+      <c r="C21" s="117"/>
+      <c r="D21" s="117"/>
       <c r="E21" s="51">
         <f>E14+E15</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F21" s="52">
         <f>F14+F15</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G21" s="53">
-        <f t="shared" ref="G21" si="7">SUM(E21:F21)</f>
-        <v>0</v>
+        <f t="shared" ref="G21:G23" si="7">SUM(E21:F21)</f>
+        <v>10</v>
       </c>
       <c r="H21" s="54">
         <f>H15</f>
@@ -3628,26 +3657,26 @@
       </c>
     </row>
     <row r="22" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A22" s="165" t="s">
+      <c r="A22" s="169" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="113"/>
-      <c r="C22" s="113"/>
-      <c r="D22" s="113"/>
+      <c r="B22" s="117"/>
+      <c r="C22" s="117"/>
+      <c r="D22" s="117"/>
       <c r="E22" s="57">
-        <f t="shared" ref="E22:L22" si="8">E16</f>
-        <v>0</v>
+        <f>E16+E17</f>
+        <v>2</v>
       </c>
       <c r="F22" s="58">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f>F16+F17</f>
+        <v>2</v>
       </c>
       <c r="G22" s="59">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>4</v>
       </c>
       <c r="H22" s="54">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="G22:L22" si="8">H16</f>
         <v>0</v>
       </c>
       <c r="I22" s="55">
@@ -3753,23 +3782,23 @@
       </c>
     </row>
     <row r="23" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A23" s="166" t="s">
+      <c r="A23" s="170" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="113"/>
-      <c r="C23" s="113"/>
-      <c r="D23" s="113"/>
+      <c r="B23" s="117"/>
+      <c r="C23" s="117"/>
+      <c r="D23" s="117"/>
       <c r="E23" s="60">
         <f t="shared" ref="E23:L23" si="9">E18</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F23" s="61">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="62">
-        <f t="shared" si="9"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>4</v>
       </c>
       <c r="H23" s="54">
         <f t="shared" si="9"/>
@@ -3878,23 +3907,23 @@
       </c>
     </row>
     <row r="24" spans="1:40" ht="19.5" customHeight="1">
-      <c r="A24" s="137" t="s">
+      <c r="A24" s="141" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="138"/>
-      <c r="C24" s="138"/>
-      <c r="D24" s="138"/>
+      <c r="B24" s="142"/>
+      <c r="C24" s="142"/>
+      <c r="D24" s="142"/>
       <c r="E24" s="108">
         <f t="shared" ref="E24:J24" si="10">SUM(E20:E23)</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F24" s="109">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G24" s="110">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H24" s="63">
         <f t="shared" si="10"/>
@@ -4076,30 +4105,30 @@
       <c r="AN25" s="1"/>
     </row>
     <row r="26" spans="1:40" ht="16.5" customHeight="1">
-      <c r="A26" s="153" t="s">
+      <c r="A26" s="157" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="116"/>
-      <c r="C26" s="116"/>
-      <c r="D26" s="116"/>
-      <c r="E26" s="116"/>
-      <c r="F26" s="116"/>
-      <c r="G26" s="116"/>
-      <c r="H26" s="116"/>
-      <c r="I26" s="116"/>
-      <c r="J26" s="116"/>
-      <c r="K26" s="116"/>
-      <c r="L26" s="116"/>
-      <c r="M26" s="116"/>
-      <c r="N26" s="116"/>
-      <c r="O26" s="116"/>
-      <c r="P26" s="116"/>
-      <c r="Q26" s="116"/>
-      <c r="R26" s="116"/>
-      <c r="S26" s="116"/>
-      <c r="T26" s="116"/>
-      <c r="U26" s="116"/>
-      <c r="V26" s="116"/>
+      <c r="B26" s="120"/>
+      <c r="C26" s="120"/>
+      <c r="D26" s="120"/>
+      <c r="E26" s="120"/>
+      <c r="F26" s="120"/>
+      <c r="G26" s="120"/>
+      <c r="H26" s="120"/>
+      <c r="I26" s="120"/>
+      <c r="J26" s="120"/>
+      <c r="K26" s="120"/>
+      <c r="L26" s="120"/>
+      <c r="M26" s="120"/>
+      <c r="N26" s="120"/>
+      <c r="O26" s="120"/>
+      <c r="P26" s="120"/>
+      <c r="Q26" s="120"/>
+      <c r="R26" s="120"/>
+      <c r="S26" s="120"/>
+      <c r="T26" s="120"/>
+      <c r="U26" s="120"/>
+      <c r="V26" s="120"/>
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
       <c r="Y26" s="1"/>
@@ -4150,16 +4179,16 @@
       <c r="Z27" s="73"/>
       <c r="AA27" s="73"/>
       <c r="AB27" s="1"/>
-      <c r="AC27" s="143"/>
-      <c r="AD27" s="144"/>
-      <c r="AE27" s="144"/>
-      <c r="AF27" s="144"/>
-      <c r="AG27" s="144"/>
-      <c r="AH27" s="144"/>
-      <c r="AI27" s="144"/>
-      <c r="AJ27" s="144"/>
-      <c r="AK27" s="144"/>
-      <c r="AL27" s="144"/>
+      <c r="AC27" s="147"/>
+      <c r="AD27" s="148"/>
+      <c r="AE27" s="148"/>
+      <c r="AF27" s="148"/>
+      <c r="AG27" s="148"/>
+      <c r="AH27" s="148"/>
+      <c r="AI27" s="148"/>
+      <c r="AJ27" s="148"/>
+      <c r="AK27" s="148"/>
+      <c r="AL27" s="148"/>
       <c r="AM27" s="3"/>
       <c r="AN27" s="3"/>
     </row>
@@ -4382,32 +4411,32 @@
       <c r="B33" s="76"/>
       <c r="C33" s="76"/>
       <c r="D33" s="1"/>
-      <c r="E33" s="152" t="s">
+      <c r="E33" s="156" t="s">
         <v>37</v>
       </c>
-      <c r="F33" s="116"/>
-      <c r="G33" s="116"/>
-      <c r="H33" s="116"/>
-      <c r="I33" s="116"/>
-      <c r="J33" s="116"/>
-      <c r="K33" s="116"/>
-      <c r="L33" s="116"/>
-      <c r="M33" s="116"/>
-      <c r="N33" s="116"/>
-      <c r="O33" s="116"/>
-      <c r="P33" s="116"/>
-      <c r="Q33" s="116"/>
+      <c r="F33" s="120"/>
+      <c r="G33" s="120"/>
+      <c r="H33" s="120"/>
+      <c r="I33" s="120"/>
+      <c r="J33" s="120"/>
+      <c r="K33" s="120"/>
+      <c r="L33" s="120"/>
+      <c r="M33" s="120"/>
+      <c r="N33" s="120"/>
+      <c r="O33" s="120"/>
+      <c r="P33" s="120"/>
+      <c r="Q33" s="120"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
-      <c r="T33" s="155" t="s">
+      <c r="T33" s="159" t="s">
         <v>38</v>
       </c>
-      <c r="U33" s="116"/>
-      <c r="V33" s="116"/>
-      <c r="W33" s="116"/>
-      <c r="X33" s="116"/>
-      <c r="Y33" s="116"/>
-      <c r="Z33" s="116"/>
+      <c r="U33" s="120"/>
+      <c r="V33" s="120"/>
+      <c r="W33" s="120"/>
+      <c r="X33" s="120"/>
+      <c r="Y33" s="120"/>
+      <c r="Z33" s="120"/>
       <c r="AA33" s="1"/>
       <c r="AB33" s="1"/>
       <c r="AC33" s="1"/>
@@ -4430,28 +4459,28 @@
       <c r="B34" s="77"/>
       <c r="C34" s="77"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="116"/>
-      <c r="F34" s="116"/>
-      <c r="G34" s="116"/>
-      <c r="H34" s="116"/>
-      <c r="I34" s="116"/>
-      <c r="J34" s="116"/>
-      <c r="K34" s="116"/>
-      <c r="L34" s="116"/>
-      <c r="M34" s="116"/>
-      <c r="N34" s="116"/>
-      <c r="O34" s="116"/>
-      <c r="P34" s="116"/>
-      <c r="Q34" s="116"/>
+      <c r="E34" s="120"/>
+      <c r="F34" s="120"/>
+      <c r="G34" s="120"/>
+      <c r="H34" s="120"/>
+      <c r="I34" s="120"/>
+      <c r="J34" s="120"/>
+      <c r="K34" s="120"/>
+      <c r="L34" s="120"/>
+      <c r="M34" s="120"/>
+      <c r="N34" s="120"/>
+      <c r="O34" s="120"/>
+      <c r="P34" s="120"/>
+      <c r="Q34" s="120"/>
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
-      <c r="T34" s="116"/>
-      <c r="U34" s="116"/>
-      <c r="V34" s="116"/>
-      <c r="W34" s="116"/>
-      <c r="X34" s="116"/>
-      <c r="Y34" s="116"/>
-      <c r="Z34" s="116"/>
+      <c r="T34" s="120"/>
+      <c r="U34" s="120"/>
+      <c r="V34" s="120"/>
+      <c r="W34" s="120"/>
+      <c r="X34" s="120"/>
+      <c r="Y34" s="120"/>
+      <c r="Z34" s="120"/>
       <c r="AA34" s="1"/>
       <c r="AB34" s="1"/>
       <c r="AC34" s="1"/>
@@ -4474,30 +4503,30 @@
       <c r="B35" s="77"/>
       <c r="C35" s="77"/>
       <c r="D35" s="1"/>
-      <c r="E35" s="116"/>
-      <c r="F35" s="116"/>
-      <c r="G35" s="116"/>
-      <c r="H35" s="116"/>
-      <c r="I35" s="116"/>
-      <c r="J35" s="116"/>
-      <c r="K35" s="116"/>
-      <c r="L35" s="116"/>
-      <c r="M35" s="116"/>
-      <c r="N35" s="116"/>
-      <c r="O35" s="116"/>
-      <c r="P35" s="116"/>
-      <c r="Q35" s="116"/>
+      <c r="E35" s="120"/>
+      <c r="F35" s="120"/>
+      <c r="G35" s="120"/>
+      <c r="H35" s="120"/>
+      <c r="I35" s="120"/>
+      <c r="J35" s="120"/>
+      <c r="K35" s="120"/>
+      <c r="L35" s="120"/>
+      <c r="M35" s="120"/>
+      <c r="N35" s="120"/>
+      <c r="O35" s="120"/>
+      <c r="P35" s="120"/>
+      <c r="Q35" s="120"/>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
-      <c r="T35" s="156" t="s">
+      <c r="T35" s="160" t="s">
         <v>41</v>
       </c>
-      <c r="U35" s="116"/>
-      <c r="V35" s="116"/>
-      <c r="W35" s="116"/>
-      <c r="X35" s="116"/>
-      <c r="Y35" s="116"/>
-      <c r="Z35" s="116"/>
+      <c r="U35" s="120"/>
+      <c r="V35" s="120"/>
+      <c r="W35" s="120"/>
+      <c r="X35" s="120"/>
+      <c r="Y35" s="120"/>
+      <c r="Z35" s="120"/>
       <c r="AA35" s="1"/>
       <c r="AB35" s="1"/>
       <c r="AC35" s="1"/>
@@ -4520,28 +4549,28 @@
       <c r="B36" s="77"/>
       <c r="C36" s="77"/>
       <c r="D36" s="1"/>
-      <c r="E36" s="116"/>
-      <c r="F36" s="116"/>
-      <c r="G36" s="116"/>
-      <c r="H36" s="116"/>
-      <c r="I36" s="116"/>
-      <c r="J36" s="116"/>
-      <c r="K36" s="116"/>
-      <c r="L36" s="116"/>
-      <c r="M36" s="116"/>
-      <c r="N36" s="116"/>
-      <c r="O36" s="116"/>
-      <c r="P36" s="116"/>
-      <c r="Q36" s="116"/>
+      <c r="E36" s="120"/>
+      <c r="F36" s="120"/>
+      <c r="G36" s="120"/>
+      <c r="H36" s="120"/>
+      <c r="I36" s="120"/>
+      <c r="J36" s="120"/>
+      <c r="K36" s="120"/>
+      <c r="L36" s="120"/>
+      <c r="M36" s="120"/>
+      <c r="N36" s="120"/>
+      <c r="O36" s="120"/>
+      <c r="P36" s="120"/>
+      <c r="Q36" s="120"/>
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
-      <c r="T36" s="116"/>
-      <c r="U36" s="116"/>
-      <c r="V36" s="116"/>
-      <c r="W36" s="116"/>
-      <c r="X36" s="116"/>
-      <c r="Y36" s="116"/>
-      <c r="Z36" s="116"/>
+      <c r="T36" s="120"/>
+      <c r="U36" s="120"/>
+      <c r="V36" s="120"/>
+      <c r="W36" s="120"/>
+      <c r="X36" s="120"/>
+      <c r="Y36" s="120"/>
+      <c r="Z36" s="120"/>
       <c r="AA36" s="1"/>
       <c r="AB36" s="1"/>
       <c r="AC36" s="1"/>
@@ -4562,19 +4591,19 @@
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
-      <c r="E37" s="116"/>
-      <c r="F37" s="116"/>
-      <c r="G37" s="116"/>
-      <c r="H37" s="116"/>
-      <c r="I37" s="116"/>
-      <c r="J37" s="116"/>
-      <c r="K37" s="116"/>
-      <c r="L37" s="116"/>
-      <c r="M37" s="116"/>
-      <c r="N37" s="116"/>
-      <c r="O37" s="116"/>
-      <c r="P37" s="116"/>
-      <c r="Q37" s="116"/>
+      <c r="E37" s="120"/>
+      <c r="F37" s="120"/>
+      <c r="G37" s="120"/>
+      <c r="H37" s="120"/>
+      <c r="I37" s="120"/>
+      <c r="J37" s="120"/>
+      <c r="K37" s="120"/>
+      <c r="L37" s="120"/>
+      <c r="M37" s="120"/>
+      <c r="N37" s="120"/>
+      <c r="O37" s="120"/>
+      <c r="P37" s="120"/>
+      <c r="Q37" s="120"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
@@ -4604,19 +4633,19 @@
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
-      <c r="E38" s="116"/>
-      <c r="F38" s="116"/>
-      <c r="G38" s="116"/>
-      <c r="H38" s="116"/>
-      <c r="I38" s="116"/>
-      <c r="J38" s="116"/>
-      <c r="K38" s="116"/>
-      <c r="L38" s="116"/>
-      <c r="M38" s="116"/>
-      <c r="N38" s="116"/>
-      <c r="O38" s="116"/>
-      <c r="P38" s="116"/>
-      <c r="Q38" s="116"/>
+      <c r="E38" s="120"/>
+      <c r="F38" s="120"/>
+      <c r="G38" s="120"/>
+      <c r="H38" s="120"/>
+      <c r="I38" s="120"/>
+      <c r="J38" s="120"/>
+      <c r="K38" s="120"/>
+      <c r="L38" s="120"/>
+      <c r="M38" s="120"/>
+      <c r="N38" s="120"/>
+      <c r="O38" s="120"/>
+      <c r="P38" s="120"/>
+      <c r="Q38" s="120"/>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
       <c r="T38" s="1"/>
@@ -13016,6 +13045,9 @@
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.17" right="0.16" top="0.23" bottom="0.19" header="0" footer="0"/>
   <pageSetup scale="78" orientation="landscape" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="G23 G20" formula="1"/>
+  </ignoredErrors>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>